<commit_message>
Replace prior reruns with researched V5 topics
</commit_message>
<xml_diff>
--- a/docs/content-v5/v5-topic-run-plan-2026-09-26.xlsx
+++ b/docs/content-v5/v5-topic-run-plan-2026-09-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run plan" sheetId="1" r:id="R9b9760b4938a4c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source analysis" sheetId="2" r:id="R0fdbcc0ae0844c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run plan" sheetId="1" r:id="R6dc143cf8b684d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source analysis" sheetId="2" r:id="R27ed5e7b861f4df1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,12 +14,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="dd mmm yyyy hh:mm"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.00"/>
+    <x:numFmt numFmtId="203" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -51,8 +52,24 @@
       <x:color rgb="FF536273"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF142334"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF142334"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF567087"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -74,6 +91,26 @@
         <x:fgColor rgb="FFFFF2CF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -81,7 +118,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -119,11 +156,78 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="V5RunPlan" displayName="V5RunPlan" ref="A5:I52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="#"/>
+    <x:tableColumn id="2" name="Post (Bangkok)"/>
+    <x:tableColumn id="3" name="Type"/>
+    <x:tableColumn id="4" name="Topic"/>
+    <x:tableColumn id="5" name="YouTube title"/>
+    <x:tableColumn id="6" name="YouTube description"/>
+    <x:tableColumn id="7" name="Brief path"/>
+    <x:tableColumn id="8" name="Source"/>
+    <x:tableColumn id="9" name="Run command"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -319,1506 +423,1521 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF17324D"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="6" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="45" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="88" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="68" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="5" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="56" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="56" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="135" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="118" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>V5 realistic video — daily run plan</x:v>
-      </x:c>
-      <x:c r="B1" s="1" t="str"/>
-      <x:c r="C1" s="1" t="str"/>
-      <x:c r="D1" s="1" t="str"/>
-      <x:c r="E1" s="1" t="str"/>
-      <x:c r="F1" s="1" t="str"/>
-      <x:c r="G1" s="1" t="str"/>
-      <x:c r="H1" s="1" t="str"/>
-      <x:c r="I1" s="1" t="str"/>
-      <x:c r="J1" s="1" t="str"/>
+      <x:c r="A1" s="26" t="str">
+        <x:v>V5 daily run plan</x:v>
+      </x:c>
+      <x:c r="B1" s="23"/>
+      <x:c r="C1" s="23"/>
+      <x:c r="D1" s="23"/>
+      <x:c r="E1" s="23"/>
+      <x:c r="F1" s="23"/>
+      <x:c r="G1" s="23"/>
+      <x:c r="H1" s="23"/>
+      <x:c r="I1" s="23"/>
+      <x:c r="J1"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="3" t="str">
-        <x:v>47 clips · 24 prior topics over 800 views · 23 new topics · 28 Sep–13 Nov 2026 · local time Asia/Bangkok</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="str"/>
-      <x:c r="C2" s="1" t="str"/>
-      <x:c r="D2" s="1" t="str"/>
-      <x:c r="E2" s="1" t="str"/>
-      <x:c r="F2" s="1" t="str"/>
-      <x:c r="G2" s="1" t="str"/>
-      <x:c r="H2" s="1" t="str"/>
-      <x:c r="I2" s="1" t="str"/>
-      <x:c r="J2" s="1" t="str"/>
+      <x:c r="A2" s="27" t="str">
+        <x:v>47 researched topics · 28 Sep–13 Nov 2026 · Asia/Bangkok</x:v>
+      </x:c>
+      <x:c r="B2" s="23"/>
+      <x:c r="C2" s="23"/>
+      <x:c r="D2" s="23"/>
+      <x:c r="E2" s="23"/>
+      <x:c r="F2" s="23"/>
+      <x:c r="G2" s="23"/>
+      <x:c r="H2" s="23"/>
+      <x:c r="I2" s="23"/>
+      <x:c r="J2"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="1"/>
-      <x:c r="B3" s="1"/>
-      <x:c r="C3" s="1"/>
-      <x:c r="D3" s="1"/>
-      <x:c r="E3" s="1"/>
-      <x:c r="F3" s="1"/>
-      <x:c r="G3" s="1"/>
-      <x:c r="H3" s="1"/>
-      <x:c r="I3" s="1"/>
-      <x:c r="J3" s="1"/>
+      <x:c r="A3" s="27" t="str">
+        <x:v>FAST_MODE=true centers and auto-approves the contradiction clip after file validation; other scenes keep normal review.</x:v>
+      </x:c>
+      <x:c r="B3" s="23"/>
+      <x:c r="C3" s="23"/>
+      <x:c r="D3" s="23"/>
+      <x:c r="E3" s="23"/>
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3"/>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="8" t="str">
+      <x:c r="A4" s="23"/>
+      <x:c r="B4" s="23"/>
+      <x:c r="C4" s="23"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="23"/>
+      <x:c r="J4"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="39" t="str">
         <x:v>#</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="str">
+      <x:c r="B5" s="39" t="str">
         <x:v>Post (Bangkok)</x:v>
       </x:c>
-      <x:c r="C4" s="8" t="str">
+      <x:c r="C5" s="39" t="str">
         <x:v>Type</x:v>
       </x:c>
-      <x:c r="D4" s="8" t="str">
+      <x:c r="D5" s="39" t="str">
         <x:v>Topic</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="E5" s="39" t="str">
         <x:v>YouTube title</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="F5" s="39" t="str">
         <x:v>YouTube description</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
-        <x:v>Previous title</x:v>
-      </x:c>
-      <x:c r="H4" s="8" t="str">
-        <x:v>Views</x:v>
-      </x:c>
-      <x:c r="I4" s="8" t="str">
+      <x:c r="G5" s="39" t="str">
         <x:v>Brief path</x:v>
       </x:c>
-      <x:c r="J4" s="8" t="str">
+      <x:c r="H5" s="39" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="I5" s="39" t="str">
         <x:v>Run command</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="9" t="n">
+      <x:c r="J5"/>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B5" s="10" t="n">
+      <x:c r="B6" s="42" t="n">
         <x:v>46293.15625</x:v>
       </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>A Runway Can Change Its Number Without Moving</x:v>
-      </x:c>
-      <x:c r="E5" s="9" t="str">
-        <x:v>This Runway’s Number Changed. The Runway Didn’t.</x:v>
-      </x:c>
-      <x:c r="F5" s="9" t="str">
-        <x:v>A painted runway number can change while the pavement stays put. Have you ever noticed an airport repaint one? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G5" s="9" t="str">
-        <x:v>A Runway Can Change Its Number Without Moving</x:v>
-      </x:c>
-      <x:c r="H5" s="11" t="n">
-        <x:v>1563</x:v>
-      </x:c>
-      <x:c r="I5" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/runway-number-change.json</x:v>
-      </x:c>
-      <x:c r="J5" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/runway-number-change.json npm run generate -- 'A Runway Can Change Its Number Without Moving' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="12" t="n">
+      <x:c r="C6" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D6" s="44" t="str">
+        <x:v>A Microwave Door Can Have Holes and Still Contain Microwaves</x:v>
+      </x:c>
+      <x:c r="E6" s="44" t="str">
+        <x:v>Your Microwave Door Is Full of Holes. Why Is That Safe?</x:v>
+      </x:c>
+      <x:c r="F6" s="44" t="str">
+        <x:v>The screen has openings you can see through, yet the oven is designed to keep microwaves inside. Had you noticed the mesh? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G6" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/microwave-door-screen.json</x:v>
+      </x:c>
+      <x:c r="H6" s="43" t="str">
+        <x:v>https://www.fda.gov/downloads/Radiation-EmittingProducts/RadiationEmittingProductsandProcedures/HomeBusinessandEntertainment/UCM119038.pdf</x:v>
+      </x:c>
+      <x:c r="I6" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/microwave-door-screen.json FAST_MODE=true npm run generate -- 'A Microwave Door Can Have Holes and Still Contain Microwaves' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J6"/>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="31" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="n">
+      <x:c r="B7" s="32" t="n">
         <x:v>46294.11111111111</x:v>
       </x:c>
-      <x:c r="C6" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D6" s="12" t="str">
+      <x:c r="C7" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D7" s="40" t="str">
         <x:v>A Pen-Cap Hole Is an Airway Safety Feature</x:v>
       </x:c>
-      <x:c r="E6" s="12" t="str">
+      <x:c r="E7" s="40" t="str">
         <x:v>The Tiny Hole in a Pen Cap Has a Serious Job</x:v>
       </x:c>
-      <x:c r="F6" s="12" t="str">
+      <x:c r="F7" s="40" t="str">
         <x:v>It looks like a stray design detail, but vented caps can meet a child-safety standard. Had you noticed that hole before? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G6" s="12" t="str"/>
-      <x:c r="H6" s="14"/>
-      <x:c r="I6" s="12" t="str">
+      <x:c r="G7" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/pen-cap-hole.json</x:v>
       </x:c>
-      <x:c r="J6" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/pen-cap-hole.json npm run generate -- 'A Pen-Cap Hole Is an Airway Safety Feature' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="28" customHeight="1">
-      <x:c r="A7" s="9" t="n">
+      <x:c r="H7" s="33" t="str">
+        <x:v>https://assets.ctfassets.net/wm1n7oady8a5/4T7UJ3QkkaTReldpTc5ORH/ad1a706f7b12e57ad28b156686aa83a6/BIC_Certificate-_Cristal_Expression_English.pdf</x:v>
+      </x:c>
+      <x:c r="I7" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/pen-cap-hole.json FAST_MODE=true npm run generate -- 'A Pen-Cap Hole Is an Airway Safety Feature' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J7"/>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="41" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B7" s="10" t="n">
+      <x:c r="B8" s="42" t="n">
         <x:v>46295.194444444445</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>A Stop Sign Is Recognizable Before You Read It</x:v>
-      </x:c>
-      <x:c r="E7" s="9" t="str">
-        <x:v>You Can Recognize This Sign Without Reading It</x:v>
-      </x:c>
-      <x:c r="F7" s="9" t="str">
-        <x:v>That familiar shape is doing work before the word is legible. Could you identify a STOP sign from the back? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G7" s="9" t="str">
-        <x:v>A Stop Sign Still Works Even If You Can't Read It</x:v>
-      </x:c>
-      <x:c r="H7" s="11" t="n">
-        <x:v>1334</x:v>
-      </x:c>
-      <x:c r="I7" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/stop-sign-shape.json</x:v>
-      </x:c>
-      <x:c r="J7" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/stop-sign-shape.json npm run generate -- 'A Stop Sign Is Recognizable Before You Read It' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="12" t="n">
+      <x:c r="C8" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D8" s="44" t="str">
+        <x:v>Three QR-Code Squares Help a Scanner Find Its Direction</x:v>
+      </x:c>
+      <x:c r="E8" s="44" t="str">
+        <x:v>Those Three QR Squares Have a Job You Probably Missed</x:v>
+      </x:c>
+      <x:c r="F8" s="44" t="str">
+        <x:v>A scanner can find a standard QR code from different directions because of those corners. Which corner did you notice first? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G8" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/qr-corner-squares.json</x:v>
+      </x:c>
+      <x:c r="H8" s="43" t="str">
+        <x:v>https://www.qrcode.com/en/about/featurePage/featurePage5.html</x:v>
+      </x:c>
+      <x:c r="I8" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/qr-corner-squares.json FAST_MODE=true npm run generate -- 'Three QR-Code Squares Help a Scanner Find Its Direction' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J8"/>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="31" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="n">
+      <x:c r="B9" s="32" t="n">
         <x:v>46296.10763888889</x:v>
       </x:c>
-      <x:c r="C8" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D8" s="12" t="str">
+      <x:c r="C9" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D9" s="40" t="str">
         <x:v>A Fire Sprinkler Waits for Heat, Not Smoke</x:v>
       </x:c>
-      <x:c r="E8" s="12" t="str">
+      <x:c r="E9" s="40" t="str">
         <x:v>Your Fire Sprinkler Ignores Smoke. Here’s What Triggers It</x:v>
       </x:c>
-      <x:c r="F8" s="12" t="str">
+      <x:c r="F9" s="40" t="str">
         <x:v>The little glass bulb waits for heat, not a whiff of smoke. Did you think every sprinkler would spray at once? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G8" s="12" t="str"/>
-      <x:c r="H8" s="14"/>
-      <x:c r="I8" s="12" t="str">
+      <x:c r="G9" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/sprinkler-glass-bulb.json</x:v>
       </x:c>
-      <x:c r="J8" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/sprinkler-glass-bulb.json npm run generate -- 'A Fire Sprinkler Waits for Heat, Not Smoke' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="9" t="n">
+      <x:c r="H9" s="33" t="str">
+        <x:v>https://apps.usfa.fema.gov/ax/sm/sm_0142.pdf</x:v>
+      </x:c>
+      <x:c r="I9" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/sprinkler-glass-bulb.json FAST_MODE=true npm run generate -- 'A Fire Sprinkler Waits for Heat, Not Smoke' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J9"/>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="41" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B9" s="10" t="n">
+      <x:c r="B10" s="42" t="n">
         <x:v>46297.177083333336</x:v>
       </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D9" s="9" t="str">
-        <x:v>Costco Checks More Than Your Receipt Total</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="str">
-        <x:v>Costco’s Exit Check Has Another Job</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="str">
-        <x:v>The person at the exit is checking more than whether you paid. Have you ever had a receipt checker catch a mistake? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G9" s="9" t="str">
-        <x:v>Costco Isn't Just Checking Whether You Paid</x:v>
-      </x:c>
-      <x:c r="H9" s="11" t="n">
-        <x:v>1229</x:v>
-      </x:c>
-      <x:c r="I9" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/costco-receipt-check.json</x:v>
-      </x:c>
-      <x:c r="J9" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/costco-receipt-check.json npm run generate -- 'Costco Checks More Than Your Receipt Total' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="12" t="n">
+      <x:c r="C10" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D10" s="44" t="str">
+        <x:v>Bumpy Curb Tiles Mark Where the Sidewalk Ends</x:v>
+      </x:c>
+      <x:c r="E10" s="44" t="str">
+        <x:v>Those Bumpy Sidewalk Tiles Are a Warning</x:v>
+      </x:c>
+      <x:c r="F10" s="44" t="str">
+        <x:v>At a flush curb, the raised pattern can make the street edge detectable underfoot. Have you felt it before crossing? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G10" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/tactile-curb-domes.json</x:v>
+      </x:c>
+      <x:c r="H10" s="43" t="str">
+        <x:v>https://www.access-board.gov/prowag/complete.html</x:v>
+      </x:c>
+      <x:c r="I10" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/tactile-curb-domes.json FAST_MODE=true npm run generate -- 'Bumpy Curb Tiles Mark Where the Sidewalk Ends' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J10"/>
+    </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="31" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B10" s="13" t="n">
+      <x:c r="B11" s="32" t="n">
         <x:v>46298.208333333336</x:v>
       </x:c>
-      <x:c r="C10" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D10" s="12" t="str">
+      <x:c r="C11" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="str">
         <x:v>Four Runway Lights Tell Pilots If They Are Too High</x:v>
       </x:c>
-      <x:c r="E10" s="12" t="str">
+      <x:c r="E11" s="40" t="str">
         <x:v>Four Lights Can Tell a Pilot They’re Too Low</x:v>
       </x:c>
-      <x:c r="F10" s="12" t="str">
+      <x:c r="F11" s="40" t="str">
         <x:v>A row of red and white lights changes with the approach angle. Have you spotted them beside a runway? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G10" s="12" t="str"/>
-      <x:c r="H10" s="14"/>
-      <x:c r="I10" s="12" t="str">
+      <x:c r="G11" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/papi-lights.json</x:v>
       </x:c>
-      <x:c r="J10" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/papi-lights.json npm run generate -- 'Four Runway Lights Tell Pilots If They Are Too High' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="9" t="n">
+      <x:c r="H11" s="33" t="str">
+        <x:v>https://www.faa.gov/about/office_org/headquarters_offices/ato/service_units/techops/navservices/lsg/papi</x:v>
+      </x:c>
+      <x:c r="I11" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/papi-lights.json FAST_MODE=true npm run generate -- 'Four Runway Lights Tell Pilots If They Are Too High' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J11"/>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="41" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B11" s="10" t="n">
+      <x:c r="B12" s="42" t="n">
         <x:v>46299.135416666664</x:v>
       </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
-        <x:v>Hidden Road Loops Can Call the Traffic Light</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str">
-        <x:v>The Traffic Light Can Sense Your Car Through the Road</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="str">
-        <x:v>Those cuts in the pavement can be part of a vehicle detector. Have you spotted one at your local intersection? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G11" s="9" t="str">
-        <x:v>Hidden Road Loops Control the Traffic Light</x:v>
-      </x:c>
-      <x:c r="H11" s="11" t="n">
-        <x:v>1211</x:v>
-      </x:c>
-      <x:c r="I11" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/traffic-light-loops.json</x:v>
-      </x:c>
-      <x:c r="J11" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/traffic-light-loops.json npm run generate -- 'Hidden Road Loops Can Call the Traffic Light' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="12" t="n">
+      <x:c r="C12" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D12" s="44" t="str">
+        <x:v>A Tire Sidewall Hides Its Manufacture Date</x:v>
+      </x:c>
+      <x:c r="E12" s="44" t="str">
+        <x:v>Your Tire Has a Birthday Hidden on Its Sidewall</x:v>
+      </x:c>
+      <x:c r="F12" s="44" t="str">
+        <x:v>Those final four DOT digits tell you when a tire was made, even if the tread looks fine. Have you checked your spare? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G12" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/tire-date-code.json</x:v>
+      </x:c>
+      <x:c r="H12" s="43" t="str">
+        <x:v>https://www.nhtsa.gov/vehicle-safety/tires</x:v>
+      </x:c>
+      <x:c r="I12" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/tire-date-code.json FAST_MODE=true npm run generate -- 'A Tire Sidewall Hides Its Manufacture Date' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J12"/>
+    </x:row>
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="31" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B12" s="13" t="n">
+      <x:c r="B13" s="32" t="n">
         <x:v>46300.208333333336</x:v>
       </x:c>
-      <x:c r="C12" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D12" s="12" t="str">
+      <x:c r="C13" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D13" s="40" t="str">
         <x:v>Runway Centerline Lights Turn Red Near the End</x:v>
       </x:c>
-      <x:c r="E12" s="12" t="str">
+      <x:c r="E13" s="40" t="str">
         <x:v>These Runway Lights Turn Red for a Reason</x:v>
       </x:c>
-      <x:c r="F12" s="12" t="str">
+      <x:c r="F13" s="40" t="str">
         <x:v>On some runways, the centerline lights change color as the end gets close. Which airport detail should we decode next? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G12" s="12" t="str"/>
-      <x:c r="H12" s="14"/>
-      <x:c r="I12" s="12" t="str">
+      <x:c r="G13" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/runway-end-lights.json</x:v>
       </x:c>
-      <x:c r="J12" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/runway-end-lights.json npm run generate -- 'Runway Centerline Lights Turn Red Near the End' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="9" t="n">
+      <x:c r="H13" s="33" t="str">
+        <x:v>https://www.faa.gov/air_traffic/publications/atpubs/aip_html/chap2_section_1.html</x:v>
+      </x:c>
+      <x:c r="I13" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/runway-end-lights.json FAST_MODE=true npm run generate -- 'Runway Centerline Lights Turn Red Near the End' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J13"/>
+    </x:row>
+    <x:row r="14" ht="42" customHeight="1">
+      <x:c r="A14" s="41" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B13" s="10" t="n">
+      <x:c r="B14" s="42" t="n">
         <x:v>46301.19097222222</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
-        <x:v>Why Some U.S. Mail Trucks Put the Driver on the Right</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="str">
-        <x:v>Why Some U.S. Mail Trucks Put Drivers on the “Wrong” Side</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="str">
-        <x:v>The steering wheel placement makes sense once you look at the mailbox. Have you seen a right-hand-drive delivery truck? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G13" s="9" t="str">
-        <x:v>America Built Mail Trucks Backwards on Purpose</x:v>
-      </x:c>
-      <x:c r="H13" s="11" t="n">
-        <x:v>1210</x:v>
-      </x:c>
-      <x:c r="I13" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/right-hand-drive-mail-trucks.json</x:v>
-      </x:c>
-      <x:c r="J13" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/right-hand-drive-mail-trucks.json npm run generate -- 'Why Some U.S. Mail Trucks Put the Driver on the Right' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="12" t="n">
+      <x:c r="C14" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D14" s="44" t="str">
+        <x:v>An Induction Stove Heats the Pan Directly</x:v>
+      </x:c>
+      <x:c r="E14" s="44" t="str">
+        <x:v>This Glass Stove Heats the Pan in a Different Way</x:v>
+      </x:c>
+      <x:c r="F14" s="44" t="str">
+        <x:v>Induction creates heat in suitable cookware rather than in a glowing burner. Would your favorite pan pass the magnet test? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G14" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/induction-pan.json</x:v>
+      </x:c>
+      <x:c r="H14" s="43" t="str">
+        <x:v>https://www.energy.gov/articles/making-switch-induction-stoves-or-cooktops</x:v>
+      </x:c>
+      <x:c r="I14" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/induction-pan.json FAST_MODE=true npm run generate -- 'An Induction Stove Heats the Pan Directly' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J14"/>
+    </x:row>
+    <x:row r="15" ht="42" customHeight="1">
+      <x:c r="A15" s="31" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B14" s="13" t="n">
+      <x:c r="B15" s="32" t="n">
         <x:v>46302.17013888889</x:v>
       </x:c>
-      <x:c r="C14" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D14" s="12" t="str">
+      <x:c r="C15" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
         <x:v>Blue and Green Airport Lights Do Different Jobs</x:v>
       </x:c>
-      <x:c r="E14" s="12" t="str">
+      <x:c r="E15" s="40" t="str">
         <x:v>Why Airport Taxiways Glow Blue and Green</x:v>
       </x:c>
-      <x:c r="F14" s="12" t="str">
+      <x:c r="F15" s="40" t="str">
         <x:v>The two colors mark different parts of a taxiway. Did you ever notice that the center and edges do not match? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G14" s="12" t="str"/>
-      <x:c r="H14" s="14"/>
-      <x:c r="I14" s="12" t="str">
+      <x:c r="G15" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/taxiway-light-colors.json</x:v>
       </x:c>
-      <x:c r="J14" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/taxiway-light-colors.json npm run generate -- 'Blue and Green Airport Lights Do Different Jobs' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="28" customHeight="1">
-      <x:c r="A15" s="9" t="n">
+      <x:c r="H15" s="33" t="str">
+        <x:v>https://www.faa.gov/air_traffic/publications/atpubs/aip_html/chap2_section_1.html</x:v>
+      </x:c>
+      <x:c r="I15" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/taxiway-light-colors.json FAST_MODE=true npm run generate -- 'Blue and Green Airport Lights Do Different Jobs' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J15"/>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="41" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B15" s="10" t="n">
+      <x:c r="B16" s="42" t="n">
         <x:v>46303.100694444445</x:v>
       </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="str">
-        <x:v>The Tiny Fuel Arrow Points to the Filler Door</x:v>
-      </x:c>
-      <x:c r="E15" s="9" t="str">
-        <x:v>The Tiny Arrow That Saves a Gas-Station U-Turn</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="str">
-        <x:v>A dashboard detail can tell you which side to pull up on. Did you know your car had this clue? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G15" s="9" t="str">
-        <x:v>Secret Fuel Arrow Points Straight to the Gas Cap</x:v>
-      </x:c>
-      <x:c r="H15" s="11" t="n">
-        <x:v>1177</x:v>
-      </x:c>
-      <x:c r="I15" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/fuel-door-arrow.json</x:v>
-      </x:c>
-      <x:c r="J15" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/fuel-door-arrow.json npm run generate -- 'The Tiny Fuel Arrow Points to the Filler Door' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="28" customHeight="1">
-      <x:c r="A16" s="12" t="n">
+      <x:c r="C16" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D16" s="44" t="str">
+        <x:v>A Plane Trail Is Mostly Ice Crystals</x:v>
+      </x:c>
+      <x:c r="E16" s="44" t="str">
+        <x:v>That White Trail Behind a Plane Isn’t Smoke</x:v>
+      </x:c>
+      <x:c r="F16" s="44" t="str">
+        <x:v>Cold air turns exhaust water into ice crystals, and humidity decides how long the trail lasts. Have you seen one spread out? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G16" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/contrail-ice.json</x:v>
+      </x:c>
+      <x:c r="H16" s="43" t="str">
+        <x:v>https://www.nasa.gov/centers-and-facilities/armstrong/nasa-partners-explore-sustainable-fuels-effects-on-aircraft-contrails/</x:v>
+      </x:c>
+      <x:c r="I16" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/contrail-ice.json FAST_MODE=true npm run generate -- 'A Plane Trail Is Mostly Ice Crystals' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J16"/>
+    </x:row>
+    <x:row r="17" ht="42" customHeight="1">
+      <x:c r="A17" s="31" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B16" s="13" t="n">
+      <x:c r="B17" s="32" t="n">
         <x:v>46304.197916666664</x:v>
       </x:c>
-      <x:c r="C16" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D16" s="12" t="str">
+      <x:c r="C17" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
         <x:v>Tiny Bars in a Tire Tread Signal Replacement</x:v>
       </x:c>
-      <x:c r="E16" s="12" t="str">
+      <x:c r="E17" s="40" t="str">
         <x:v>Your Tire Hides a Replacement Warning</x:v>
       </x:c>
-      <x:c r="F16" s="12" t="str">
+      <x:c r="F17" s="40" t="str">
         <x:v>The small raised bar in a tire groove becomes a clue as tread wears down. Have you checked yours lately? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G16" s="12" t="str"/>
-      <x:c r="H16" s="14"/>
-      <x:c r="I16" s="12" t="str">
+      <x:c r="G17" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/tire-wear-bars.json</x:v>
       </x:c>
-      <x:c r="J16" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/tire-wear-bars.json npm run generate -- 'Tiny Bars in a Tire Tread Signal Replacement' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="28" customHeight="1">
-      <x:c r="A17" s="9" t="n">
+      <x:c r="H17" s="33" t="str">
+        <x:v>https://www.nhtsa.gov/vehicle-safety/tires</x:v>
+      </x:c>
+      <x:c r="I17" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/tire-wear-bars.json FAST_MODE=true npm run generate -- 'Tiny Bars in a Tire Tread Signal Replacement' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J17"/>
+    </x:row>
+    <x:row r="18" ht="42" customHeight="1">
+      <x:c r="A18" s="41" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B17" s="10" t="n">
+      <x:c r="B18" s="42" t="n">
         <x:v>46305.13888888889</x:v>
       </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="str">
-        <x:v>Wind Makes the Same Air Feel Colder</x:v>
-      </x:c>
-      <x:c r="E17" s="9" t="str">
-        <x:v>Same Temperature. Why Does It Feel So Much Colder?</x:v>
-      </x:c>
-      <x:c r="F17" s="9" t="str">
-        <x:v>The thermometer can stay the same while your skin loses heat faster. What is the windiest cold day you remember? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G17" s="9" t="str">
-        <x:v>Same Temperature. Completely Different Chill.</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="n">
-        <x:v>1167</x:v>
-      </x:c>
-      <x:c r="I17" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/wind-chill.json</x:v>
-      </x:c>
-      <x:c r="J17" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/wind-chill.json npm run generate -- 'Wind Makes the Same Air Feel Colder' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="28" customHeight="1">
-      <x:c r="A18" s="12" t="n">
+      <x:c r="C18" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D18" s="44" t="str">
+        <x:v>The Two Buttons on a GFCI Outlet Guard Against Shock</x:v>
+      </x:c>
+      <x:c r="E18" s="44" t="str">
+        <x:v>Those Two Outlet Buttons Aren’t Just for Resetting</x:v>
+      </x:c>
+      <x:c r="F18" s="44" t="str">
+        <x:v>A GFCI watches for current escaping its intended path and shuts power off. Did you know what TEST actually checks? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G18" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/gfci-current-leak.json</x:v>
+      </x:c>
+      <x:c r="H18" s="43" t="str">
+        <x:v>https://www.cpsc.gov/s3fs-public/518.pdf</x:v>
+      </x:c>
+      <x:c r="I18" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/gfci-current-leak.json FAST_MODE=true npm run generate -- 'The Two Buttons on a GFCI Outlet Guard Against Shock' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J18"/>
+    </x:row>
+    <x:row r="19" ht="42" customHeight="1">
+      <x:c r="A19" s="31" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B18" s="13" t="n">
+      <x:c r="B19" s="32" t="n">
         <x:v>46306.083333333336</x:v>
       </x:c>
-      <x:c r="C18" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D18" s="12" t="str">
+      <x:c r="C19" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D19" s="40" t="str">
         <x:v>The Gap in a Bridge Lets It Move</x:v>
       </x:c>
-      <x:c r="E18" s="12" t="str">
+      <x:c r="E19" s="40" t="str">
         <x:v>That Gap in the Bridge Is Doing More Than You Think</x:v>
       </x:c>
-      <x:c r="F18" s="12" t="str">
+      <x:c r="F19" s="40" t="str">
         <x:v>Bridges need room for temperature-driven movement. Do you notice the small bump when your car crosses a joint? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G18" s="12" t="str"/>
-      <x:c r="H18" s="14"/>
-      <x:c r="I18" s="12" t="str">
+      <x:c r="G19" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/bridge-expansion-joints.json</x:v>
       </x:c>
-      <x:c r="J18" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/bridge-expansion-joints.json npm run generate -- 'The Gap in a Bridge Lets It Move' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="28" customHeight="1">
-      <x:c r="A19" s="9" t="n">
+      <x:c r="H19" s="33" t="str">
+        <x:v>https://www.fhwa.dot.gov/bridge/pubs/hif17019.pdf</x:v>
+      </x:c>
+      <x:c r="I19" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/bridge-expansion-joints.json FAST_MODE=true npm run generate -- 'The Gap in a Bridge Lets It Move' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J19"/>
+    </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="41" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="n">
+      <x:c r="B20" s="42" t="n">
         <x:v>46307.145833333336</x:v>
       </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>A U.S. Shelf Price May Exclude Sales Tax</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:v>That Shelf Price May Not Be What You Pay</x:v>
-      </x:c>
-      <x:c r="F19" s="9" t="str">
-        <x:v>In places such as Washington State, tax can appear only at checkout unless the shelf price says it is included. Does your local shop show tax upfront? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G19" s="9" t="str">
-        <x:v>America's Price Tags Often Hide the Final Price</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="n">
-        <x:v>1141</x:v>
-      </x:c>
-      <x:c r="I19" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/sales-tax-shelf-price.json</x:v>
-      </x:c>
-      <x:c r="J19" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/sales-tax-shelf-price.json npm run generate -- 'A U.S. Shelf Price May Exclude Sales Tax' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="28" customHeight="1">
-      <x:c r="A20" s="12" t="n">
+      <x:c r="C20" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D20" s="44" t="str">
+        <x:v>A Smoke Alarm Needs Replacement Even If It Still Beeps</x:v>
+      </x:c>
+      <x:c r="E20" s="44" t="str">
+        <x:v>That Smoke Alarm Can Expire While It Still Looks Fine</x:v>
+      </x:c>
+      <x:c r="F20" s="44" t="str">
+        <x:v>The date on the back matters even when the front looks normal. How old is the oldest alarm in your home? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G20" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/smoke-alarm-age.json</x:v>
+      </x:c>
+      <x:c r="H20" s="43" t="str">
+        <x:v>https://www.usfa.fema.gov/prevention/home-fires/prepare-for-fire/smoke-alarms/</x:v>
+      </x:c>
+      <x:c r="I20" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/smoke-alarm-age.json FAST_MODE=true npm run generate -- 'A Smoke Alarm Needs Replacement Even If It Still Beeps' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J20"/>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="31" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B20" s="13" t="n">
+      <x:c r="B21" s="32" t="n">
         <x:v>46308.083333333336</x:v>
       </x:c>
-      <x:c r="C20" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D20" s="12" t="str">
+      <x:c r="C21" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D21" s="40" t="str">
         <x:v>A Guardrail End Can Flatten Its Own Rail</x:v>
       </x:c>
-      <x:c r="E20" s="12" t="str">
+      <x:c r="E21" s="40" t="str">
         <x:v>A Guardrail Can Crush Itself to Slow a Crash</x:v>
       </x:c>
-      <x:c r="F20" s="12" t="str">
+      <x:c r="F21" s="40" t="str">
         <x:v>Some guardrail ends deform to absorb energy in a head-on impact. Had you noticed the special end piece? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G20" s="12" t="str"/>
-      <x:c r="H20" s="14"/>
-      <x:c r="I20" s="12" t="str">
+      <x:c r="G21" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/guardrail-terminal.json</x:v>
       </x:c>
-      <x:c r="J20" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/guardrail-terminal.json npm run generate -- 'A Guardrail End Can Flatten Its Own Rail' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="28" customHeight="1">
-      <x:c r="A21" s="9" t="n">
+      <x:c r="H21" s="33" t="str">
+        <x:v>https://highways.fhwa.dot.gov/safety/rwd/reduce-crash-severity/guardrail-101</x:v>
+      </x:c>
+      <x:c r="I21" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/guardrail-terminal.json FAST_MODE=true npm run generate -- 'A Guardrail End Can Flatten Its Own Rail' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J21"/>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="41" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B21" s="10" t="n">
+      <x:c r="B22" s="42" t="n">
         <x:v>46309.15625</x:v>
       </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>Those Red Spheres Outside Target Are Bollards</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="str">
-        <x:v>Those Giant Red Balls Outside Target Have a Job</x:v>
-      </x:c>
-      <x:c r="F21" s="9" t="str">
-        <x:v>They are a striking part of some Target entrances, but they are not only decoration. What did you think they were for? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G21" s="9" t="str">
-        <x:v>Target's Giant Red Balls Are Actually Safety Equipment</x:v>
-      </x:c>
-      <x:c r="H21" s="11" t="n">
-        <x:v>1131</x:v>
-      </x:c>
-      <x:c r="I21" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/target-bollards.json</x:v>
-      </x:c>
-      <x:c r="J21" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/target-bollards.json npm run generate -- 'Those Red Spheres Outside Target Are Bollards' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="28" customHeight="1">
-      <x:c r="A22" s="12" t="n">
+      <x:c r="C22" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D22" s="44" t="str">
+        <x:v>Tiny Glass Beads Make Road Paint Shine at Night</x:v>
+      </x:c>
+      <x:c r="E22" s="44" t="str">
+        <x:v>Road Paint Has Tiny Glass Beads Hidden in It</x:v>
+      </x:c>
+      <x:c r="F22" s="44" t="str">
+        <x:v>Those beads send headlight light back toward drivers, but rain can change the effect. Have you noticed a wet road look different? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G22" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/road-paint-beads.json</x:v>
+      </x:c>
+      <x:c r="H22" s="43" t="str">
+        <x:v>https://www.fhwa.dot.gov/hfl/partnerships/all_weather_pavement/hif13004/chap01.cfm</x:v>
+      </x:c>
+      <x:c r="I22" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/road-paint-beads.json FAST_MODE=true npm run generate -- 'Tiny Glass Beads Make Road Paint Shine at Night' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J22"/>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="31" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B22" s="13" t="n">
+      <x:c r="B23" s="32" t="n">
         <x:v>46310.135416666664</x:v>
       </x:c>
-      <x:c r="C22" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D22" s="12" t="str">
+      <x:c r="C23" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D23" s="40" t="str">
         <x:v>Those Straight Road Cuts Tell Concrete Where to Crack</x:v>
       </x:c>
-      <x:c r="E22" s="12" t="str">
+      <x:c r="E23" s="40" t="str">
         <x:v>Road Crews Cut Concrete So It Cracks There</x:v>
       </x:c>
-      <x:c r="F22" s="12" t="str">
+      <x:c r="F23" s="40" t="str">
         <x:v>A straight joint gives a concrete slab a planned place to crack. Did you think the cuts were only decorative? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G22" s="12" t="str"/>
-      <x:c r="H22" s="14"/>
-      <x:c r="I22" s="12" t="str">
+      <x:c r="G23" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/concrete-road-joints.json</x:v>
       </x:c>
-      <x:c r="J22" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/concrete-road-joints.json npm run generate -- 'Those Straight Road Cuts Tell Concrete Where to Crack' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="28" customHeight="1">
-      <x:c r="A23" s="9" t="n">
+      <x:c r="H23" s="33" t="str">
+        <x:v>https://www.fhwa.dot.gov/pavement/ta504030.pdf</x:v>
+      </x:c>
+      <x:c r="I23" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/concrete-road-joints.json FAST_MODE=true npm run generate -- 'Those Straight Road Cuts Tell Concrete Where to Crack' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J23"/>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="41" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B23" s="10" t="n">
+      <x:c r="B24" s="42" t="n">
         <x:v>46311.131944444445</x:v>
       </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
-        <x:v>Costco Keeps Its Hot-Dog Combo at $1.50</x:v>
-      </x:c>
-      <x:c r="E23" s="9" t="str">
-        <x:v>Costco’s $1.50 Hot Dog Still Feels Impossible</x:v>
-      </x:c>
-      <x:c r="F23" s="9" t="str">
-        <x:v>The hot dog and soda combo remains a memorable Costco food-court offer. Is this the first thing you buy after shopping? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G23" s="9" t="str">
-        <x:v>Costco's $1.50 Hot Dog Is a Marketing Weapon</x:v>
-      </x:c>
-      <x:c r="H23" s="11" t="n">
-        <x:v>1118</x:v>
-      </x:c>
-      <x:c r="I23" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/costco-hot-dog.json</x:v>
-      </x:c>
-      <x:c r="J23" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/costco-hot-dog.json npm run generate -- 'Costco Keeps Its Hot-Dog Combo at $1.50' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="28" customHeight="1">
-      <x:c r="A24" s="12" t="n">
+      <x:c r="C24" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D24" s="44" t="str">
+        <x:v>Red and Green Wing Lights Show an Airplane’s Direction</x:v>
+      </x:c>
+      <x:c r="E24" s="44" t="str">
+        <x:v>Those Red and Green Plane Lights Give Away Its Direction</x:v>
+      </x:c>
+      <x:c r="F24" s="44" t="str">
+        <x:v>The wingtip colors are assigned by side, so their pattern helps reveal orientation. Could you tell which way this plane is facing? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G24" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/airplane-position-lights.json</x:v>
+      </x:c>
+      <x:c r="H24" s="43" t="str">
+        <x:v>https://www.faa.gov/sites/faa.gov/files/regulations_policies/handbooks_manuals/aviation/airplane_handbook/12_afh_ch11.pdf</x:v>
+      </x:c>
+      <x:c r="I24" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/airplane-position-lights.json FAST_MODE=true npm run generate -- 'Red and Green Wing Lights Show an Airplane’s Direction' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J24"/>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B24" s="13" t="n">
+      <x:c r="B25" s="32" t="n">
         <x:v>46312.18402777778</x:v>
       </x:c>
-      <x:c r="C24" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D24" s="12" t="str">
+      <x:c r="C25" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D25" s="40" t="str">
         <x:v>A Water Tower Uses Height to Push Water</x:v>
       </x:c>
-      <x:c r="E24" s="12" t="str">
+      <x:c r="E25" s="40" t="str">
         <x:v>Why Your Water Tower Is So High</x:v>
       </x:c>
-      <x:c r="F24" s="12" t="str">
+      <x:c r="F25" s="40" t="str">
         <x:v>Once water is up in a tower, gravity can help move it through the pipes. Is there a water tower near you? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G24" s="12" t="str"/>
-      <x:c r="H24" s="14"/>
-      <x:c r="I24" s="12" t="str">
+      <x:c r="G25" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/water-tower-pressure.json</x:v>
       </x:c>
-      <x:c r="J24" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/water-tower-pressure.json npm run generate -- 'A Water Tower Uses Height to Push Water' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="9" t="n">
+      <x:c r="H25" s="33" t="str">
+        <x:v>https://pubs.usgs.gov/gip/7000045/report.pdf</x:v>
+      </x:c>
+      <x:c r="I25" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/water-tower-pressure.json FAST_MODE=true npm run generate -- 'A Water Tower Uses Height to Push Water' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J25"/>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="41" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B25" s="10" t="n">
+      <x:c r="B26" s="42" t="n">
         <x:v>46313.083333333336</x:v>
       </x:c>
-      <x:c r="C25" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="str">
-        <x:v>A Toll Road Can Bill a Car Without a Booth</x:v>
-      </x:c>
-      <x:c r="E25" s="9" t="str">
-        <x:v>No Toll Booth? You Can Still Get a Bill</x:v>
-      </x:c>
-      <x:c r="F25" s="9" t="str">
-        <x:v>A Florida toll road can record a plate and send the owner a bill. Have you ever missed the moment a toll was charged? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G25" s="9" t="str">
-        <x:v>No Toll Booth. Still a Bill.</x:v>
-      </x:c>
-      <x:c r="H25" s="11" t="n">
-        <x:v>1094</x:v>
-      </x:c>
-      <x:c r="I25" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/toll-by-plate.json</x:v>
-      </x:c>
-      <x:c r="J25" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/toll-by-plate.json npm run generate -- 'A Toll Road Can Bill a Car Without a Booth' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="28" customHeight="1">
-      <x:c r="A26" s="12" t="n">
+      <x:c r="C26" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D26" s="44" t="str">
+        <x:v>The Stones Under Train Tracks Hold the Geometry</x:v>
+      </x:c>
+      <x:c r="E26" s="44" t="str">
+        <x:v>Those Track Stones Are Doing More Than Filling Space</x:v>
+      </x:c>
+      <x:c r="F26" s="44" t="str">
+        <x:v>Railway ballast helps hold the track’s shape, and maintenance machines move it back into place. Had you noticed how much stone is there? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G26" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/railway-ballast.json</x:v>
+      </x:c>
+      <x:c r="H26" s="43" t="str">
+        <x:v>https://www.networkrail.co.uk/our-work/looking-after-the-railway/track/</x:v>
+      </x:c>
+      <x:c r="I26" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/railway-ballast.json FAST_MODE=true npm run generate -- 'The Stones Under Train Tracks Hold the Geometry' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J26"/>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="31" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B26" s="13" t="n">
+      <x:c r="B27" s="32" t="n">
         <x:v>46314.10763888889</x:v>
       </x:c>
-      <x:c r="C26" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D26" s="12" t="str">
+      <x:c r="C27" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
         <x:v>A Storm Drain May Lead Straight to a River</x:v>
       </x:c>
-      <x:c r="E26" s="12" t="str">
+      <x:c r="E27" s="40" t="str">
         <x:v>That Street Drain May Lead Straight to a River</x:v>
       </x:c>
-      <x:c r="F26" s="12" t="str">
+      <x:c r="F27" s="40" t="str">
         <x:v>In a separate storm-sewer system, runoff can reach waterways without a treatment plant. Where does rain go on your street? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G26" s="12" t="str"/>
-      <x:c r="H26" s="14"/>
-      <x:c r="I26" s="12" t="str">
+      <x:c r="G27" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/storm-drain-route.json</x:v>
       </x:c>
-      <x:c r="J26" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/storm-drain-route.json npm run generate -- 'A Storm Drain May Lead Straight to a River' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="28" customHeight="1">
-      <x:c r="A27" s="9" t="n">
+      <x:c r="H27" s="33" t="str">
+        <x:v>https://www.epa.gov/nutrientpollution/sources-and-solutions-stormwater</x:v>
+      </x:c>
+      <x:c r="I27" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/storm-drain-route.json FAST_MODE=true npm run generate -- 'A Storm Drain May Lead Straight to a River' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J27"/>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="41" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B27" s="10" t="n">
+      <x:c r="B28" s="42" t="n">
         <x:v>46315.125</x:v>
       </x:c>
-      <x:c r="C27" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D27" s="9" t="str">
-        <x:v>Exit 145 Can Be a Distance Clue</x:v>
-      </x:c>
-      <x:c r="E27" s="9" t="str">
-        <x:v>Exit 145 Is Hiding a Distance Clue</x:v>
-      </x:c>
-      <x:c r="F27" s="9" t="str">
-        <x:v>On many U.S. interstates, the exit number helps locate you along the route. Do you use exit numbers to judge a drive? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G27" s="9" t="str">
-        <x:v>Exit 145 Can Tell You How Far You've Driven</x:v>
-      </x:c>
-      <x:c r="H27" s="11" t="n">
-        <x:v>1090</x:v>
-      </x:c>
-      <x:c r="I27" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/mile-based-exits.json</x:v>
-      </x:c>
-      <x:c r="J27" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/mile-based-exits.json npm run generate -- 'Exit 145 Can Be a Distance Clue' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="28" customHeight="1">
-      <x:c r="A28" s="12" t="n">
+      <x:c r="C28" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D28" s="44" t="str">
+        <x:v>A Popcorn Kernel Turns Itself Inside Out</x:v>
+      </x:c>
+      <x:c r="E28" s="44" t="str">
+        <x:v>A Popcorn Kernel Explodes Inside Out</x:v>
+      </x:c>
+      <x:c r="F28" s="44" t="str">
+        <x:v>The puff is starch pushed outward when pressure breaks the hard shell. Have you ever watched one pop in slow motion? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G28" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/popcorn-steam.json</x:v>
+      </x:c>
+      <x:c r="H28" s="43" t="str">
+        <x:v>https://www.nal.usda.gov/exhibits/speccoll/exhibits/show/popcorn/how-does-popcorn-pop-</x:v>
+      </x:c>
+      <x:c r="I28" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/popcorn-steam.json FAST_MODE=true npm run generate -- 'A Popcorn Kernel Turns Itself Inside Out' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J28"/>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="31" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B28" s="13" t="n">
+      <x:c r="B29" s="32" t="n">
         <x:v>46316.194444444445</x:v>
       </x:c>
-      <x:c r="C28" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D28" s="12" t="str">
+      <x:c r="C29" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D29" s="40" t="str">
         <x:v>The Last Barcode Digit Checks the Others</x:v>
       </x:c>
-      <x:c r="E28" s="12" t="str">
+      <x:c r="E29" s="40" t="str">
         <x:v>Your Barcode’s Last Digit Checks the Rest</x:v>
       </x:c>
-      <x:c r="F28" s="12" t="str">
+      <x:c r="F29" s="40" t="str">
         <x:v>The final digit of a product code has a quiet error-checking job. Did you think every digit identified the product? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G28" s="12" t="str"/>
-      <x:c r="H28" s="14"/>
-      <x:c r="I28" s="12" t="str">
+      <x:c r="G29" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/barcode-check-digit.json</x:v>
       </x:c>
-      <x:c r="J28" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/barcode-check-digit.json npm run generate -- 'The Last Barcode Digit Checks the Others' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="28" customHeight="1">
-      <x:c r="A29" s="9" t="n">
+      <x:c r="H29" s="33" t="str">
+        <x:v>https://www.gs1.org/services/check-digit-calculator</x:v>
+      </x:c>
+      <x:c r="I29" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/barcode-check-digit.json FAST_MODE=true npm run generate -- 'The Last Barcode Digit Checks the Others' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J29"/>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="41" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B29" s="10" t="n">
+      <x:c r="B30" s="42" t="n">
         <x:v>46317.13888888889</x:v>
       </x:c>
-      <x:c r="C29" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
-        <x:v>Escalator Brushes Help Keep Feet Clear</x:v>
-      </x:c>
-      <x:c r="E29" s="9" t="str">
-        <x:v>Those Escalator Brushes Aren’t for Your Shoes</x:v>
-      </x:c>
-      <x:c r="F29" s="9" t="str">
-        <x:v>The brush beside the moving steps has a safety role. What did you think it was there for? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G29" s="9" t="str">
-        <x:v>Escalator Brushes Are Safety Guards, Not Shoe Cleaners</x:v>
-      </x:c>
-      <x:c r="H29" s="11" t="n">
-        <x:v>1067</x:v>
-      </x:c>
-      <x:c r="I29" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/escalator-brushes.json</x:v>
-      </x:c>
-      <x:c r="J29" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/escalator-brushes.json npm run generate -- 'Escalator Brushes Help Keep Feet Clear' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="28" customHeight="1">
-      <x:c r="A30" s="12" t="n">
+      <x:c r="C30" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D30" s="44" t="str">
+        <x:v>The Horizon Moon Looks Bigger Without Growing</x:v>
+      </x:c>
+      <x:c r="E30" s="44" t="str">
+        <x:v>The Moon Isn’t Growing Near the Horizon</x:v>
+      </x:c>
+      <x:c r="F30" s="44" t="str">
+        <x:v>The low Moon looks huge, but matched photos show a different story. Have you ever checked it with your own camera? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G30" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/moon-horizon-illusion.json</x:v>
+      </x:c>
+      <x:c r="H30" s="43" t="str">
+        <x:v>https://science.nasa.gov/solar-system/moon/the-moon-illusion-why-does-the-moon-look-so-big-sometimes/</x:v>
+      </x:c>
+      <x:c r="I30" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/moon-horizon-illusion.json FAST_MODE=true npm run generate -- 'The Horizon Moon Looks Bigger Without Growing' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J30"/>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="31" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B30" s="13" t="n">
+      <x:c r="B31" s="32" t="n">
         <x:v>46318.208333333336</x:v>
       </x:c>
-      <x:c r="C30" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D30" s="12" t="str">
+      <x:c r="C31" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D31" s="40" t="str">
         <x:v>A Mail Barcode Can Track One Envelope</x:v>
       </x:c>
-      <x:c r="E30" s="12" t="str">
+      <x:c r="E31" s="40" t="str">
         <x:v>That Barcode on Your Letter Does More Than Sort It</x:v>
       </x:c>
-      <x:c r="F30" s="12" t="str">
+      <x:c r="F31" s="40" t="str">
         <x:v>USPS Intelligent Mail bars can carry routing and tracking information. Have you ever noticed the tiny bars below an address? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G30" s="12" t="str"/>
-      <x:c r="H30" s="14"/>
-      <x:c r="I30" s="12" t="str">
+      <x:c r="G31" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/postal-intelligent-barcode.json</x:v>
       </x:c>
-      <x:c r="J30" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/postal-intelligent-barcode.json npm run generate -- 'A Mail Barcode Can Track One Envelope' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="28" customHeight="1">
-      <x:c r="A31" s="9" t="n">
+      <x:c r="H31" s="33" t="str">
+        <x:v>https://pe.usps.com/text/dmm300/204.htm</x:v>
+      </x:c>
+      <x:c r="I31" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/postal-intelligent-barcode.json FAST_MODE=true npm run generate -- 'A Mail Barcode Can Track One Envelope' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J31"/>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="41" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B31" s="10" t="n">
+      <x:c r="B32" s="42" t="n">
         <x:v>46319.17361111111</x:v>
       </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D31" s="9" t="str">
-        <x:v>A Cut Apple Changes After the Knife Leaves</x:v>
-      </x:c>
-      <x:c r="E31" s="9" t="str">
-        <x:v>Your Apple Changes After the Knife Leaves</x:v>
-      </x:c>
-      <x:c r="F31" s="9" t="str">
-        <x:v>The slice keeps reacting after you set the knife down. Do you use lemon juice or just eat it before it browns? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G31" s="9" t="str">
-        <x:v>The Apple Changes After the Knife Leaves</x:v>
-      </x:c>
-      <x:c r="H31" s="11" t="n">
-        <x:v>1038</x:v>
-      </x:c>
-      <x:c r="I31" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/apple-browning.json</x:v>
-      </x:c>
-      <x:c r="J31" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/apple-browning.json npm run generate -- 'A Cut Apple Changes After the Knife Leaves' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="28" customHeight="1">
-      <x:c r="A32" s="12" t="n">
+      <x:c r="C32" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D32" s="44" t="str">
+        <x:v>Water Can Boil Below 100°C in the Mountains</x:v>
+      </x:c>
+      <x:c r="E32" s="44" t="str">
+        <x:v>Water Can Boil While Staying Cooler Than You Think</x:v>
+      </x:c>
+      <x:c r="F32" s="44" t="str">
+        <x:v>Higher altitude changes the boiling point; a pressure cooker changes pressure the other way. Have you cooked in the mountains? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G32" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/high-altitude-boiling.json</x:v>
+      </x:c>
+      <x:c r="H32" s="43" t="str">
+        <x:v>https://www.fsis.usda.gov/food-safety/safe-food-handling-and-preparation/food-safety-basics/high-altitude-cooking</x:v>
+      </x:c>
+      <x:c r="I32" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/high-altitude-boiling.json FAST_MODE=true npm run generate -- 'Water Can Boil Below 100°C in the Mountains' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J32"/>
+    </x:row>
+    <x:row r="33" ht="42" customHeight="1">
+      <x:c r="A33" s="31" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B32" s="13" t="n">
+      <x:c r="B33" s="32" t="n">
         <x:v>46320.15277777778</x:v>
       </x:c>
-      <x:c r="C32" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D32" s="12" t="str">
+      <x:c r="C33" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D33" s="40" t="str">
         <x:v>The Blue Ribbon on a $100 Bill Is Woven In</x:v>
       </x:c>
-      <x:c r="E32" s="12" t="str">
+      <x:c r="E33" s="40" t="str">
         <x:v>The Blue Strip on a $100 Bill Isn’t Printed</x:v>
       </x:c>
-      <x:c r="F32" s="12" t="str">
+      <x:c r="F33" s="40" t="str">
         <x:v>The blue ribbon is woven into the note, and its images move when you tilt it. Have you seen that effect in person? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G32" s="12" t="str"/>
-      <x:c r="H32" s="14"/>
-      <x:c r="I32" s="12" t="str">
+      <x:c r="G33" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/hundred-dollar-ribbon.json</x:v>
       </x:c>
-      <x:c r="J32" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/hundred-dollar-ribbon.json npm run generate -- 'The Blue Ribbon on a $100 Bill Is Woven In' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="9" t="n">
+      <x:c r="H33" s="33" t="str">
+        <x:v>https://www.uscurrency.gov/educational-materials/decoding-dollars-100</x:v>
+      </x:c>
+      <x:c r="I33" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/hundred-dollar-ribbon.json FAST_MODE=true npm run generate -- 'The Blue Ribbon on a $100 Bill Is Woven In' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J33"/>
+    </x:row>
+    <x:row r="34" ht="42" customHeight="1">
+      <x:c r="A34" s="41" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B33" s="10" t="n">
+      <x:c r="B34" s="42" t="n">
         <x:v>46321.125</x:v>
       </x:c>
-      <x:c r="C33" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>Frost-Free Freezers Heat Their Coils on Purpose</x:v>
-      </x:c>
-      <x:c r="E33" s="9" t="str">
-        <x:v>Your Freezer Turns On a Heater. On Purpose.</x:v>
-      </x:c>
-      <x:c r="F33" s="9" t="str">
-        <x:v>A frost-free freezer briefly uses heat where ice builds up. Did you expect a heater inside something meant to stay cold? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G33" s="9" t="str">
-        <x:v>Frost-Free Freezers Fire Heaters On Purpose</x:v>
-      </x:c>
-      <x:c r="H33" s="11" t="n">
-        <x:v>1018</x:v>
-      </x:c>
-      <x:c r="I33" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/freezer-defrost-heater.json</x:v>
-      </x:c>
-      <x:c r="J33" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/freezer-defrost-heater.json npm run generate -- 'Frost-Free Freezers Heat Their Coils on Purpose' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="28" customHeight="1">
-      <x:c r="A34" s="12" t="n">
+      <x:c r="C34" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D34" s="44" t="str">
+        <x:v>A Fire Extinguisher Gauge Can Reveal a Problem</x:v>
+      </x:c>
+      <x:c r="E34" s="44" t="str">
+        <x:v>That Fire Extinguisher Gauge Could Be Warning You</x:v>
+      </x:c>
+      <x:c r="F34" s="44" t="str">
+        <x:v>Pressure is one check, but the hose and body matter too. Do you know where your extinguisher is? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G34" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/fire-extinguisher-pressure.json</x:v>
+      </x:c>
+      <x:c r="H34" s="43" t="str">
+        <x:v>https://www.usfa.fema.gov/prevention/home-fires/prepare-for-fire/fire-extinguishers/</x:v>
+      </x:c>
+      <x:c r="I34" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/fire-extinguisher-pressure.json FAST_MODE=true npm run generate -- 'A Fire Extinguisher Gauge Can Reveal a Problem' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J34"/>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="31" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B34" s="13" t="n">
+      <x:c r="B35" s="32" t="n">
         <x:v>46322.131944444445</x:v>
       </x:c>
-      <x:c r="C34" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D34" s="12" t="str">
+      <x:c r="C35" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D35" s="40" t="str">
         <x:v>The Raised Rim Protects a Coin’s Design</x:v>
       </x:c>
-      <x:c r="E34" s="12" t="str">
+      <x:c r="E35" s="40" t="str">
         <x:v>The Rim of a Coin Takes the Wear First</x:v>
       </x:c>
-      <x:c r="F34" s="12" t="str">
+      <x:c r="F35" s="40" t="str">
         <x:v>That raised edge helps protect the design on the face. Which coin detail have you never thought to inspect? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G34" s="12" t="str"/>
-      <x:c r="H34" s="14"/>
-      <x:c r="I34" s="12" t="str">
+      <x:c r="G35" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/coin-rim.json</x:v>
       </x:c>
-      <x:c r="J34" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/coin-rim.json npm run generate -- 'The Raised Rim Protects a Coin’s Design' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="28" customHeight="1">
-      <x:c r="A35" s="9" t="n">
+      <x:c r="H35" s="33" t="str">
+        <x:v>https://www.usmint.gov/learn/collecting-basics/anatomy-of-a-coin</x:v>
+      </x:c>
+      <x:c r="I35" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/coin-rim.json FAST_MODE=true npm run generate -- 'The Raised Rim Protects a Coin’s Design' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J35"/>
+    </x:row>
+    <x:row r="36" ht="42" customHeight="1">
+      <x:c r="A36" s="41" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B35" s="10" t="n">
+      <x:c r="B36" s="42" t="n">
         <x:v>46323.131944444445</x:v>
       </x:c>
-      <x:c r="C35" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D35" s="9" t="str">
-        <x:v>Road Reflector Colors Carry Direction Cues</x:v>
-      </x:c>
-      <x:c r="E35" s="9" t="str">
-        <x:v>Road Reflectors Can Warn You’re Going the Wrong Way</x:v>
-      </x:c>
-      <x:c r="F35" s="9" t="str">
-        <x:v>A reflector may send a different color back from the opposite direction. Have you noticed red reflectors facing oncoming traffic? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G35" s="9" t="str">
-        <x:v>Road Reflectors Speak in Colour</x:v>
-      </x:c>
-      <x:c r="H35" s="11" t="n">
-        <x:v>1003</x:v>
-      </x:c>
-      <x:c r="I35" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/road-reflector-colors.json</x:v>
-      </x:c>
-      <x:c r="J35" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/road-reflector-colors.json npm run generate -- 'Road Reflector Colors Carry Direction Cues' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="28" customHeight="1">
-      <x:c r="A36" s="12" t="n">
+      <x:c r="C36" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D36" s="44" t="str">
+        <x:v>USB-C Works Upside Down for a Reason</x:v>
+      </x:c>
+      <x:c r="E36" s="44" t="str">
+        <x:v>The USB-C Flip Works Because of What’s Inside</x:v>
+      </x:c>
+      <x:c r="F36" s="44" t="str">
+        <x:v>The plug’s orientation can reverse, but the connected signals still need the right path. Did you ever miss the old one-way plug? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G36" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/usb-c-flip.json</x:v>
+      </x:c>
+      <x:c r="H36" s="43" t="str">
+        <x:v>https://usb.org/usb-type-cr-cable-and-connector-specification</x:v>
+      </x:c>
+      <x:c r="I36" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/usb-c-flip.json FAST_MODE=true npm run generate -- 'USB-C Works Upside Down for a Reason' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J36"/>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="31" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B36" s="13" t="n">
+      <x:c r="B37" s="32" t="n">
         <x:v>46324.177083333336</x:v>
       </x:c>
-      <x:c r="C36" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D36" s="12" t="str">
+      <x:c r="C37" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D37" s="40" t="str">
         <x:v>Ordinary Foil Works on Either Side</x:v>
       </x:c>
-      <x:c r="E36" s="12" t="str">
+      <x:c r="E37" s="40" t="str">
         <x:v>The Shiny Side of Foil Doesn’t Matter—Except When It Does</x:v>
       </x:c>
-      <x:c r="F36" s="12" t="str">
+      <x:c r="F37" s="40" t="str">
         <x:v>Ordinary foil works either way, but specialty non-stick foil is different. Which side do you usually put against food? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G36" s="12" t="str"/>
-      <x:c r="H36" s="14"/>
-      <x:c r="I36" s="12" t="str">
+      <x:c r="G37" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/foil-two-sides.json</x:v>
       </x:c>
-      <x:c r="J36" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/foil-two-sides.json npm run generate -- 'Ordinary Foil Works on Either Side' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="28" customHeight="1">
-      <x:c r="A37" s="9" t="n">
+      <x:c r="H37" s="33" t="str">
+        <x:v>https://www.reynoldsbrands.com/tips-and-how-tos/aluminum-foil-guide</x:v>
+      </x:c>
+      <x:c r="I37" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/foil-two-sides.json FAST_MODE=true npm run generate -- 'Ordinary Foil Works on Either Side' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J37"/>
+    </x:row>
+    <x:row r="38" ht="42" customHeight="1">
+      <x:c r="A38" s="41" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B37" s="10" t="n">
+      <x:c r="B38" s="42" t="n">
         <x:v>46325.19097222222</x:v>
       </x:c>
-      <x:c r="C37" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D37" s="9" t="str">
-        <x:v>Amazon Stores Different Products in the Same Pod</x:v>
-      </x:c>
-      <x:c r="E37" s="9" t="str">
-        <x:v>Amazon’s Shelves Look Random for a Reason</x:v>
-      </x:c>
-      <x:c r="F37" s="9" t="str">
-        <x:v>Mixing products in robotic storage pods can solve a traffic problem inside the warehouse. Would you have organized them by product instead? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G37" s="9" t="str">
-        <x:v>Amazon Makes Warehouses Faster by Making Shelves Look Random</x:v>
-      </x:c>
-      <x:c r="H37" s="11" t="n">
-        <x:v>971</x:v>
-      </x:c>
-      <x:c r="I37" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/amazon-stow-pods.json</x:v>
-      </x:c>
-      <x:c r="J37" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/amazon-stow-pods.json npm run generate -- 'Amazon Stores Different Products in the Same Pod' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="28" customHeight="1">
-      <x:c r="A38" s="12" t="n">
+      <x:c r="C38" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D38" s="44" t="str">
+        <x:v>A Second Rainbow Reverses the Color Order</x:v>
+      </x:c>
+      <x:c r="E38" s="44" t="str">
+        <x:v>A Double Rainbow Hides a Color Reversal</x:v>
+      </x:c>
+      <x:c r="F38" s="44" t="str">
+        <x:v>The outer bow forms after an extra reflection in raindrops—and its colors flip. Have you spotted the reversal? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G38" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/double-rainbow.json</x:v>
+      </x:c>
+      <x:c r="H38" s="43" t="str">
+        <x:v>https://www.nesdis.noaa.gov/about/k-12-education/optical-phenomena/what-causes-rainbow</x:v>
+      </x:c>
+      <x:c r="I38" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/double-rainbow.json FAST_MODE=true npm run generate -- 'A Second Rainbow Reverses the Color Order' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J38"/>
+    </x:row>
+    <x:row r="39" ht="42" customHeight="1">
+      <x:c r="A39" s="31" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B38" s="13" t="n">
+      <x:c r="B39" s="32" t="n">
         <x:v>46326.180555555555</x:v>
       </x:c>
-      <x:c r="C38" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D38" s="12" t="str">
+      <x:c r="C39" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D39" s="40" t="str">
         <x:v>Dishwasher Rinse Aid Helps Water Slide Away</x:v>
       </x:c>
-      <x:c r="E38" s="12" t="str">
+      <x:c r="E39" s="40" t="str">
         <x:v>The Dishwasher Additive That Makes Water Slip Away</x:v>
       </x:c>
-      <x:c r="F38" s="12" t="str">
+      <x:c r="F39" s="40" t="str">
         <x:v>Rinse aid helps droplets slide off dishes so they dry better. Do your glasses still come out wet? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G38" s="12" t="str"/>
-      <x:c r="H38" s="14"/>
-      <x:c r="I38" s="12" t="str">
+      <x:c r="G39" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/dishwasher-rinse-aid.json</x:v>
       </x:c>
-      <x:c r="J38" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/dishwasher-rinse-aid.json npm run generate -- 'Dishwasher Rinse Aid Helps Water Slide Away' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="28" customHeight="1">
-      <x:c r="A39" s="9" t="n">
+      <x:c r="H39" s="33" t="str">
+        <x:v>https://www.bosch-home.com/us/experience-bosch/heart-of-the-home/innovations/dishwashers/tips-for-achieving-dryer-dishes</x:v>
+      </x:c>
+      <x:c r="I39" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/dishwasher-rinse-aid.json FAST_MODE=true npm run generate -- 'Dishwasher Rinse Aid Helps Water Slide Away' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J39"/>
+    </x:row>
+    <x:row r="40" ht="42" customHeight="1">
+      <x:c r="A40" s="41" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B39" s="10" t="n">
+      <x:c r="B40" s="42" t="n">
         <x:v>46327.086805555555</x:v>
       </x:c>
-      <x:c r="C39" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D39" s="9" t="str">
-        <x:v>The Water Outside Your Glass Came From the Air</x:v>
-      </x:c>
-      <x:c r="E39" s="9" t="str">
-        <x:v>Your Cold Drink Isn’t Leaking. So Why Is It Wet?</x:v>
-      </x:c>
-      <x:c r="F39" s="9" t="str">
-        <x:v>The droplets on the outside may have come from the air around you. Does your glass leave a ring on the table? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G39" s="9" t="str">
-        <x:v>Your Drink Isn’t Leaking. The Air Is Getting Wet.</x:v>
-      </x:c>
-      <x:c r="H39" s="11" t="n">
-        <x:v>925</x:v>
-      </x:c>
-      <x:c r="I39" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/cold-glass-condensation.json</x:v>
-      </x:c>
-      <x:c r="J39" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/cold-glass-condensation.json npm run generate -- 'The Water Outside Your Glass Came From the Air' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="28" customHeight="1">
-      <x:c r="A40" s="12" t="n">
+      <x:c r="C40" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D40" s="44" t="str">
+        <x:v>Sunset Light Travels Through More Air and Loses Blue</x:v>
+      </x:c>
+      <x:c r="E40" s="44" t="str">
+        <x:v>Sunset Turns Red Because Blue Light Takes a Detour</x:v>
+      </x:c>
+      <x:c r="F40" s="44" t="str">
+        <x:v>The low Sun’s light crosses more air, changing what reaches your eyes. Was your last sunset orange or deep red? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G40" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/red-sunset.json</x:v>
+      </x:c>
+      <x:c r="H40" s="43" t="str">
+        <x:v>https://www.nesdis.noaa.gov/about/k-12-education/atmosphere/why-the-sky-blue</x:v>
+      </x:c>
+      <x:c r="I40" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/red-sunset.json FAST_MODE=true npm run generate -- 'Sunset Light Travels Through More Air and Loses Blue' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J40"/>
+    </x:row>
+    <x:row r="41" ht="42" customHeight="1">
+      <x:c r="A41" s="31" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B40" s="13" t="n">
+      <x:c r="B41" s="32" t="n">
         <x:v>46328.09722222222</x:v>
       </x:c>
-      <x:c r="C40" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D40" s="12" t="str">
+      <x:c r="C41" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D41" s="40" t="str">
         <x:v>Small Wingtip Fins Reduce a Bigger Drag</x:v>
       </x:c>
-      <x:c r="E40" s="12" t="str">
+      <x:c r="E41" s="40" t="str">
         <x:v>Those Tiny Wing Tips Can Save a Lot of Fuel</x:v>
       </x:c>
-      <x:c r="F40" s="12" t="str">
+      <x:c r="F41" s="40" t="str">
         <x:v>Winglets change the airflow at the tip and can reduce drag. Have you noticed how different aircraft shape theirs? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G40" s="12" t="str"/>
-      <x:c r="H40" s="14"/>
-      <x:c r="I40" s="12" t="str">
+      <x:c r="G41" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/airplane-winglets.json</x:v>
       </x:c>
-      <x:c r="J40" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/airplane-winglets.json npm run generate -- 'Small Wingtip Fins Reduce a Bigger Drag' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="28" customHeight="1">
-      <x:c r="A41" s="9" t="n">
+      <x:c r="H41" s="33" t="str">
+        <x:v>https://www1.grc.nasa.gov/beginners-guide-to-aeronautics/winglets/</x:v>
+      </x:c>
+      <x:c r="I41" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/airplane-winglets.json FAST_MODE=true npm run generate -- 'Small Wingtip Fins Reduce a Bigger Drag' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J41"/>
+    </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42" s="41" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B41" s="10" t="n">
+      <x:c r="B42" s="42" t="n">
         <x:v>46329.100694444445</x:v>
       </x:c>
-      <x:c r="C41" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D41" s="9" t="str">
-        <x:v>Maple Syrup Needs Far More Sap Than You Think</x:v>
-      </x:c>
-      <x:c r="E41" s="9" t="str">
-        <x:v>One Bottle of Maple Syrup Starts With HOW Much Sap?</x:v>
-      </x:c>
-      <x:c r="F41" s="9" t="str">
-        <x:v>A small bottle can require a surprising amount of maple sap. What would your guess be before seeing the ratio? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G41" s="9" t="str">
-        <x:v>A Lot of Sap for a Little Syrup</x:v>
-      </x:c>
-      <x:c r="H41" s="11" t="n">
-        <x:v>911</x:v>
-      </x:c>
-      <x:c r="I41" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/maple-sap-ratio.json</x:v>
-      </x:c>
-      <x:c r="J41" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/maple-sap-ratio.json npm run generate -- 'Maple Syrup Needs Far More Sap Than You Think' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="28" customHeight="1">
-      <x:c r="A42" s="12" t="n">
+      <x:c r="C42" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D42" s="44" t="str">
+        <x:v>Yellow Leaves Were Hiding Their Color All Summer</x:v>
+      </x:c>
+      <x:c r="E42" s="44" t="str">
+        <x:v>That Yellow Leaf Wasn’t Suddenly Painted Yellow</x:v>
+      </x:c>
+      <x:c r="F42" s="44" t="str">
+        <x:v>As green chlorophyll fades, other pigments show through—and reds can form differently. Which fall color do you notice first? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G42" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/autumn-leaf-pigments.json</x:v>
+      </x:c>
+      <x:c r="H42" s="43" t="str">
+        <x:v>https://www.fs.usda.gov/Internet/FSE_DOCUMENTS/stelprd3817419.pdf</x:v>
+      </x:c>
+      <x:c r="I42" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/autumn-leaf-pigments.json FAST_MODE=true npm run generate -- 'Yellow Leaves Were Hiding Their Color All Summer' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J42"/>
+    </x:row>
+    <x:row r="43" ht="42" customHeight="1">
+      <x:c r="A43" s="31" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="B42" s="13" t="n">
+      <x:c r="B43" s="32" t="n">
         <x:v>46330.145833333336</x:v>
       </x:c>
-      <x:c r="C42" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D42" s="12" t="str">
+      <x:c r="C43" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D43" s="40" t="str">
         <x:v>Invisible Window Coating Can Block Heat</x:v>
       </x:c>
-      <x:c r="E42" s="12" t="str">
+      <x:c r="E43" s="40" t="str">
         <x:v>This Invisible Window Layer Blocks Heat</x:v>
       </x:c>
-      <x:c r="F42" s="12" t="str">
+      <x:c r="F43" s="40" t="str">
         <x:v>Some clear windows carry a thin coating that changes how heat passes through. Can you tell which of your windows has it? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G42" s="12" t="str"/>
-      <x:c r="H42" s="14"/>
-      <x:c r="I42" s="12" t="str">
+      <x:c r="G43" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/low-e-window.json</x:v>
       </x:c>
-      <x:c r="J42" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/low-e-window.json npm run generate -- 'Invisible Window Coating Can Block Heat' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="28" customHeight="1">
-      <x:c r="A43" s="9" t="n">
+      <x:c r="H43" s="33" t="str">
+        <x:v>https://www.energy.gov/energysaver/window-types-and-technologies</x:v>
+      </x:c>
+      <x:c r="I43" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/low-e-window.json FAST_MODE=true npm run generate -- 'Invisible Window Coating Can Block Heat' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J43"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="41" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B43" s="10" t="n">
+      <x:c r="B44" s="42" t="n">
         <x:v>46331.18402777778</x:v>
       </x:c>
-      <x:c r="C43" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D43" s="9" t="str">
-        <x:v>A Tiny Hole Helps Stop the Fuel Nozzle</x:v>
-      </x:c>
-      <x:c r="E43" s="9" t="str">
-        <x:v>The Gas Pump’s Tiny Hole Knows When to Stop</x:v>
-      </x:c>
-      <x:c r="F43" s="9" t="str">
-        <x:v>That click at the pump comes from a small sensing opening in the nozzle. Had you ever looked for it? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G43" s="9" t="str">
-        <x:v>Your Gas Pump Stops Because of a Tiny Hole You Never Notice</x:v>
-      </x:c>
-      <x:c r="H43" s="11" t="n">
-        <x:v>885</x:v>
-      </x:c>
-      <x:c r="I43" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/gas-nozzle-shutoff.json</x:v>
-      </x:c>
-      <x:c r="J43" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/gas-nozzle-shutoff.json npm run generate -- 'A Tiny Hole Helps Stop the Fuel Nozzle' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="28" customHeight="1">
-      <x:c r="A44" s="12" t="n">
+      <x:c r="C44" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D44" s="44" t="str">
+        <x:v>A Geyser Erupts After Pressure Suddenly Drops</x:v>
+      </x:c>
+      <x:c r="E44" s="44" t="str">
+        <x:v>A Geyser’s Biggest Burst Starts With a Pressure Drop</x:v>
+      </x:c>
+      <x:c r="F44" s="44" t="str">
+        <x:v>A narrow underground pathway and hot water set up the eruption. Have you ever seen one in person? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G44" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/geyser-pressure.json</x:v>
+      </x:c>
+      <x:c r="H44" s="43" t="str">
+        <x:v>https://www.usgs.gov/observatories/yvo/news/yellowstones-active-hydrothermal-system-whats-hot-water</x:v>
+      </x:c>
+      <x:c r="I44" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/geyser-pressure.json FAST_MODE=true npm run generate -- 'A Geyser Erupts After Pressure Suddenly Drops' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J44"/>
+    </x:row>
+    <x:row r="45" ht="42" customHeight="1">
+      <x:c r="A45" s="31" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B44" s="13" t="n">
+      <x:c r="B45" s="32" t="n">
         <x:v>46332.114583333336</x:v>
       </x:c>
-      <x:c r="C44" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D44" s="12" t="str">
+      <x:c r="C45" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D45" s="40" t="str">
         <x:v>One Ripening Fruit Can Change Its Neighbors</x:v>
       </x:c>
-      <x:c r="E44" s="12" t="str">
+      <x:c r="E45" s="40" t="str">
         <x:v>One Fruit Can Make the Others Ripen Faster</x:v>
       </x:c>
-      <x:c r="F44" s="12" t="str">
+      <x:c r="F45" s="40" t="str">
         <x:v>Ethylene from some fruit can change its neighbors in a produce bowl. Which fruit always seems to ripen first at your place? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G44" s="12" t="str"/>
-      <x:c r="H44" s="14"/>
-      <x:c r="I44" s="12" t="str">
+      <x:c r="G45" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/fruit-ethylene.json</x:v>
       </x:c>
-      <x:c r="J44" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/fruit-ethylene.json npm run generate -- 'One Ripening Fruit Can Change Its Neighbors' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="28" customHeight="1">
-      <x:c r="A45" s="9" t="n">
+      <x:c r="H45" s="33" t="str">
+        <x:v>https://www.fna.usda.gov/fs/produce-safety/storage</x:v>
+      </x:c>
+      <x:c r="I45" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/fruit-ethylene.json FAST_MODE=true npm run generate -- 'One Ripening Fruit Can Change Its Neighbors' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J45"/>
+    </x:row>
+    <x:row r="46" ht="42" customHeight="1">
+      <x:c r="A46" s="41" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B45" s="10" t="n">
+      <x:c r="B46" s="42" t="n">
         <x:v>46333.145833333336</x:v>
       </x:c>
-      <x:c r="C45" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D45" s="9" t="str">
-        <x:v>Popcorn Is a Major Movie-Theater Revenue Line</x:v>
-      </x:c>
-      <x:c r="E45" s="9" t="str">
-        <x:v>Movie Tickets Aren’t the Theater’s Whole Business</x:v>
-      </x:c>
-      <x:c r="F45" s="9" t="str">
-        <x:v>AMC reports food and drinks as a major revenue line alongside admissions. Are you a popcorn person or a bring-nothing person? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G45" s="9" t="str">
-        <x:v>Movie Theaters Need Your Popcorn More Than You Think</x:v>
-      </x:c>
-      <x:c r="H45" s="11" t="n">
-        <x:v>875</x:v>
-      </x:c>
-      <x:c r="I45" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/theater-concessions.json</x:v>
-      </x:c>
-      <x:c r="J45" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/theater-concessions.json npm run generate -- 'Popcorn Is a Major Movie-Theater Revenue Line' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="28" customHeight="1">
-      <x:c r="A46" s="12" t="n">
+      <x:c r="C46" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D46" s="44" t="str">
+        <x:v>Ocean Waves Can Grow Far From the Beach</x:v>
+      </x:c>
+      <x:c r="E46" s="44" t="str">
+        <x:v>The Wind That Made This Wave May Be Far Away</x:v>
+      </x:c>
+      <x:c r="F46" s="44" t="str">
+        <x:v>Open-water distance and blowing time help waves grow before they arrive. Is your beach usually calm or rough? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G46" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/wind-wave-fetch.json</x:v>
+      </x:c>
+      <x:c r="H46" s="43" t="str">
+        <x:v>https://vos.noaa.gov/MWL/apr_06/waves.shtml</x:v>
+      </x:c>
+      <x:c r="I46" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/wind-wave-fetch.json FAST_MODE=true npm run generate -- 'Ocean Waves Can Grow Far From the Beach' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J46"/>
+    </x:row>
+    <x:row r="47" ht="42" customHeight="1">
+      <x:c r="A47" s="31" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B46" s="13" t="n">
+      <x:c r="B47" s="32" t="n">
         <x:v>46334.12152777778</x:v>
       </x:c>
-      <x:c r="C46" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D46" s="12" t="str">
+      <x:c r="C47" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D47" s="40" t="str">
         <x:v>Ice Floats Because Freezing Spreads Water Apart</x:v>
       </x:c>
-      <x:c r="E46" s="12" t="str">
+      <x:c r="E47" s="40" t="str">
         <x:v>Ice Breaks the Usual Rule When It Freezes</x:v>
       </x:c>
-      <x:c r="F46" s="12" t="str">
+      <x:c r="F47" s="40" t="str">
         <x:v>Water spreads into a more open structure when it freezes, helping ordinary ice float. Have you noticed how much of an ice cube stays submerged? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G46" s="12" t="str"/>
-      <x:c r="H46" s="14"/>
-      <x:c r="I46" s="12" t="str">
+      <x:c r="G47" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/ice-floats.json</x:v>
       </x:c>
-      <x:c r="J46" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/ice-floats.json npm run generate -- 'Ice Floats Because Freezing Spreads Water Apart' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="28" customHeight="1">
-      <x:c r="A47" s="9" t="n">
+      <x:c r="H47" s="33" t="str">
+        <x:v>https://www.usgs.gov/water-science-school/science/water-density</x:v>
+      </x:c>
+      <x:c r="I47" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/ice-floats.json FAST_MODE=true npm run generate -- 'Ice Floats Because Freezing Spreads Water Apart' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J47"/>
+    </x:row>
+    <x:row r="48" ht="42" customHeight="1">
+      <x:c r="A48" s="41" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B47" s="10" t="n">
+      <x:c r="B48" s="42" t="n">
         <x:v>46335.18402777778</x:v>
       </x:c>
-      <x:c r="C47" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D47" s="9" t="str">
-        <x:v>The Highway Warns Drivers Through Their Tires</x:v>
-      </x:c>
-      <x:c r="E47" s="9" t="str">
-        <x:v>Your Tires Hit These Grooves for a Reason</x:v>
-      </x:c>
-      <x:c r="F47" s="9" t="str">
-        <x:v>The buzz at the edge of a highway is an intentional warning. Have those grooves ever caught your attention? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G47" s="9" t="str">
-        <x:v>The Highway Is Literally Designed to Yell at Your Tires</x:v>
-      </x:c>
-      <x:c r="H47" s="11" t="n">
-        <x:v>870</x:v>
-      </x:c>
-      <x:c r="I47" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/rumble-strips.json</x:v>
-      </x:c>
-      <x:c r="J47" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/rumble-strips.json npm run generate -- 'The Highway Warns Drivers Through Their Tires' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="28" customHeight="1">
-      <x:c r="A48" s="12" t="n">
+      <x:c r="C48" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D48" s="44" t="str">
+        <x:v>Ocean Water Acts Like a Color Filter</x:v>
+      </x:c>
+      <x:c r="E48" s="44" t="str">
+        <x:v>The Ocean Isn’t Blue Just Because It Reflects the Sky</x:v>
+      </x:c>
+      <x:c r="F48" s="44" t="str">
+        <x:v>Water filters sunlight, while particles can change the color you see. What color is the water near you? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G48" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/ocean-blue-filter.json</x:v>
+      </x:c>
+      <x:c r="H48" s="43" t="str">
+        <x:v>https://oceanservice.noaa.gov/facts/oceanblue.html</x:v>
+      </x:c>
+      <x:c r="I48" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/ocean-blue-filter.json FAST_MODE=true npm run generate -- 'Ocean Water Acts Like a Color Filter' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J48"/>
+    </x:row>
+    <x:row r="49" ht="42" customHeight="1">
+      <x:c r="A49" s="31" t="n">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="B48" s="13" t="n">
+      <x:c r="B49" s="32" t="n">
         <x:v>46336.177083333336</x:v>
       </x:c>
-      <x:c r="C48" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D48" s="12" t="str">
+      <x:c r="C49" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D49" s="40" t="str">
         <x:v>Lightning and Thunder Start Together</x:v>
       </x:c>
-      <x:c r="E48" s="12" t="str">
+      <x:c r="E49" s="40" t="str">
         <x:v>Lightning and Thunder Happen Together. So Why the Delay?</x:v>
       </x:c>
-      <x:c r="F48" s="12" t="str">
+      <x:c r="F49" s="40" t="str">
         <x:v>The flash arrives before the sound even though they begin in the same event. What was the longest delay you have counted? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G48" s="12" t="str"/>
-      <x:c r="H48" s="14"/>
-      <x:c r="I48" s="12" t="str">
+      <x:c r="G49" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/lightning-thunder-delay.json</x:v>
       </x:c>
-      <x:c r="J48" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/lightning-thunder-delay.json npm run generate -- 'Lightning and Thunder Start Together' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="28" customHeight="1">
-      <x:c r="A49" s="9" t="n">
+      <x:c r="H49" s="33" t="str">
+        <x:v>https://www.weather.gov/safety/lightning-science-thunder</x:v>
+      </x:c>
+      <x:c r="I49" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/lightning-thunder-delay.json FAST_MODE=true npm run generate -- 'Lightning and Thunder Start Together' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J49"/>
+    </x:row>
+    <x:row r="50" ht="42" customHeight="1">
+      <x:c r="A50" s="41" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B49" s="10" t="n">
+      <x:c r="B50" s="42" t="n">
         <x:v>46337.163194444445</x:v>
       </x:c>
-      <x:c r="C49" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D49" s="9" t="str">
-        <x:v>The Fizz Waits Inside a Sealed Soda</x:v>
-      </x:c>
-      <x:c r="E49" s="9" t="str">
-        <x:v>The Fizz Was Inside Before You Opened It</x:v>
-      </x:c>
-      <x:c r="F49" s="9" t="str">
-        <x:v>The bubbles appear after pressure drops, but the gas was already dissolved. Do you hear the hiss before you see the fizz? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G49" s="9" t="str">
-        <x:v>The Fizz Was Waiting for You to Open It</x:v>
-      </x:c>
-      <x:c r="H49" s="11" t="n">
-        <x:v>855</x:v>
-      </x:c>
-      <x:c r="I49" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/soda-carbonation.json</x:v>
-      </x:c>
-      <x:c r="J49" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/soda-carbonation.json npm run generate -- 'The Fizz Waits Inside a Sealed Soda' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="28" customHeight="1">
-      <x:c r="A50" s="12" t="n">
+      <x:c r="C50" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D50" s="44" t="str">
+        <x:v>A Paler Pavement Can Stay Cooler in the Sun</x:v>
+      </x:c>
+      <x:c r="E50" s="44" t="str">
+        <x:v>That Lighter Pavement Can Change the Heat Underfoot</x:v>
+      </x:c>
+      <x:c r="F50" s="44" t="str">
+        <x:v>Some pavement designs reflect more Sun or cool by evaporation. Have you felt the difference between surfaces? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G50" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/cool-pavement.json</x:v>
+      </x:c>
+      <x:c r="H50" s="43" t="str">
+        <x:v>https://www.epa.gov/heatislands/using-cool-pavements-reduce-heat-islands</x:v>
+      </x:c>
+      <x:c r="I50" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/cool-pavement.json FAST_MODE=true npm run generate -- 'A Paler Pavement Can Stay Cooler in the Sun' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J50"/>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="A51" s="31" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="B50" s="13" t="n">
+      <x:c r="B51" s="32" t="n">
         <x:v>46338.11111111111</x:v>
       </x:c>
-      <x:c r="C50" s="15" t="str">
-        <x:v>New research</x:v>
-      </x:c>
-      <x:c r="D50" s="12" t="str">
+      <x:c r="C51" s="33" t="str">
+        <x:v>New research (existing)</x:v>
+      </x:c>
+      <x:c r="D51" s="40" t="str">
         <x:v>Road Salt Makes Ice Melt Below Freezing</x:v>
       </x:c>
-      <x:c r="E50" s="12" t="str">
+      <x:c r="E51" s="40" t="str">
         <x:v>Salt Doesn’t Just Melt Ice—It Changes the Freeze Point</x:v>
       </x:c>
-      <x:c r="F50" s="12" t="str">
+      <x:c r="F51" s="40" t="str">
         <x:v>Salt forms brine that can loosen ice from a road. Did you think it was simply heating the pavement? #TellMeWhyyyyyy #Shorts</x:v>
       </x:c>
-      <x:c r="G50" s="12" t="str"/>
-      <x:c r="H50" s="14"/>
-      <x:c r="I50" s="12" t="str">
+      <x:c r="G51" s="33" t="str">
         <x:v>content/v5/batch-2026-09-26/road-salt-brine.json</x:v>
       </x:c>
-      <x:c r="J50" s="12" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/road-salt-brine.json npm run generate -- 'Road Salt Makes Ice Melt Below Freezing' 'Use the reviewed brief'</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="28" customHeight="1">
-      <x:c r="A51" s="9" t="n">
+      <x:c r="H51" s="33" t="str">
+        <x:v>https://pubs.usgs.gov/wri/2001/wri01_4260/</x:v>
+      </x:c>
+      <x:c r="I51" s="33" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/road-salt-brine.json FAST_MODE=true npm run generate -- 'Road Salt Makes Ice Melt Below Freezing' 'Use the reviewed brief'</x:v>
+      </x:c>
+      <x:c r="J51"/>
+    </x:row>
+    <x:row r="52" ht="42" customHeight="1">
+      <x:c r="A52" s="41" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B51" s="10" t="n">
+      <x:c r="B52" s="42" t="n">
         <x:v>46339.177083333336</x:v>
       </x:c>
-      <x:c r="C51" s="9" t="str">
-        <x:v>Prior &gt;800</x:v>
-      </x:c>
-      <x:c r="D51" s="9" t="str">
-        <x:v>Costco Built a Poultry Supply Chain</x:v>
-      </x:c>
-      <x:c r="E51" s="9" t="str">
-        <x:v>Costco Built a Chicken Operation for Its Rotisserie Birds</x:v>
-      </x:c>
-      <x:c r="F51" s="9" t="str">
-        <x:v>Costco’s poultry operation helps supply its rotisserie chickens. Did you know the company was involved before the birds reached the store? #TellMeWhyyyyyy #Shorts</x:v>
-      </x:c>
-      <x:c r="G51" s="9" t="str">
-        <x:v>Costco Built a Supply Chain to Protect a $4.99 Chicken</x:v>
-      </x:c>
-      <x:c r="H51" s="11" t="n">
-        <x:v>849</x:v>
-      </x:c>
-      <x:c r="I51" s="9" t="str">
-        <x:v>content/v5/batch-2026-09-26/costco-poultry-supply.json</x:v>
-      </x:c>
-      <x:c r="J51" s="9" t="str">
-        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/costco-poultry-supply.json npm run generate -- 'Costco Built a Poultry Supply Chain' 'Use the reviewed brief'</x:v>
+      <x:c r="C52" s="43" t="str">
+        <x:v>New research (added)</x:v>
+      </x:c>
+      <x:c r="D52" s="44" t="str">
+        <x:v>Sleet Bounces but Freezing Rain Glazes the Ground</x:v>
+      </x:c>
+      <x:c r="E52" s="44" t="str">
+        <x:v>Two Kinds of Winter Rain Behave Completely Differently</x:v>
+      </x:c>
+      <x:c r="F52" s="44" t="str">
+        <x:v>One refreezes before landing; the other freezes on contact. Have you ever heard sleet bounce off a window? #TellMeWhyyyyyy #Shorts</x:v>
+      </x:c>
+      <x:c r="G52" s="43" t="str">
+        <x:v>content/v5/batch-2026-09-26/sleet-vs-freezing-rain.json</x:v>
+      </x:c>
+      <x:c r="H52" s="43" t="str">
+        <x:v>https://www.weather.gov/iwx/sleetvsfreezingrain</x:v>
+      </x:c>
+      <x:c r="I52" s="43" t="str">
+        <x:v>CONTENT_ENGINE_VERSION=v5 CONTENT_BRIEF_PATH=content/v5/batch-2026-09-26/sleet-vs-freezing-rain.json FAST_MODE=true npm run generate -- 'Sleet Bounces but Freezing Rain Glazes the Ground' 'Use the reviewed brief'</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca69a94e254a49f2"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Schedule two V5 clips per day
</commit_message>
<xml_diff>
--- a/docs/content-v5/v5-topic-run-plan-2026-09-26.xlsx
+++ b/docs/content-v5/v5-topic-run-plan-2026-09-26.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run plan" sheetId="1" r:id="R6dc143cf8b684d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source analysis" sheetId="2" r:id="R27ed5e7b861f4df1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run plan" sheetId="1" r:id="R824caba41c4e42b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source analysis" sheetId="2" r:id="Rdf09fa06e033495e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -456,7 +456,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="27" t="str">
-        <x:v>47 researched topics · 28 Sep–13 Nov 2026 · Asia/Bangkok</x:v>
+        <x:v>47 researched topics · 2 clips/day · 28 Sep–21 Oct 2026 · Asia/Bangkok</x:v>
       </x:c>
       <x:c r="B2" s="23"/>
       <x:c r="C2" s="23"/>
@@ -528,8 +528,8 @@
       <x:c r="A6" s="41" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="42" t="n">
-        <x:v>46293.15625</x:v>
+      <x:c r="B6" s="35" t="n">
+        <x:v>46293.09375</x:v>
       </x:c>
       <x:c r="C6" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -559,7 +559,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="32" t="n">
-        <x:v>46294.11111111111</x:v>
+        <x:v>46293.180555555555</x:v>
       </x:c>
       <x:c r="C7" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -588,8 +588,8 @@
       <x:c r="A8" s="41" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="42" t="n">
-        <x:v>46295.194444444445</x:v>
+      <x:c r="B8" s="35" t="n">
+        <x:v>46294.100694444445</x:v>
       </x:c>
       <x:c r="C8" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -619,7 +619,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B9" s="32" t="n">
-        <x:v>46296.10763888889</x:v>
+        <x:v>46294.15972222222</x:v>
       </x:c>
       <x:c r="C9" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -648,8 +648,8 @@
       <x:c r="A10" s="41" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="42" t="n">
-        <x:v>46297.177083333336</x:v>
+      <x:c r="B10" s="35" t="n">
+        <x:v>46295.086805555555</x:v>
       </x:c>
       <x:c r="C10" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -679,7 +679,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="32" t="n">
-        <x:v>46298.208333333336</x:v>
+        <x:v>46295.15972222222</x:v>
       </x:c>
       <x:c r="C11" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -708,8 +708,8 @@
       <x:c r="A12" s="41" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B12" s="42" t="n">
-        <x:v>46299.135416666664</x:v>
+      <x:c r="B12" s="35" t="n">
+        <x:v>46296.10763888889</x:v>
       </x:c>
       <x:c r="C12" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -739,7 +739,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B13" s="32" t="n">
-        <x:v>46300.208333333336</x:v>
+        <x:v>46296.177083333336</x:v>
       </x:c>
       <x:c r="C13" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -768,8 +768,8 @@
       <x:c r="A14" s="41" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B14" s="42" t="n">
-        <x:v>46301.19097222222</x:v>
+      <x:c r="B14" s="35" t="n">
+        <x:v>46297.100694444445</x:v>
       </x:c>
       <x:c r="C14" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -799,7 +799,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B15" s="32" t="n">
-        <x:v>46302.17013888889</x:v>
+        <x:v>46297.19097222222</x:v>
       </x:c>
       <x:c r="C15" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -828,8 +828,8 @@
       <x:c r="A16" s="41" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B16" s="42" t="n">
-        <x:v>46303.100694444445</x:v>
+      <x:c r="B16" s="35" t="n">
+        <x:v>46298.086805555555</x:v>
       </x:c>
       <x:c r="C16" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -859,7 +859,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B17" s="32" t="n">
-        <x:v>46304.197916666664</x:v>
+        <x:v>46298.17013888889</x:v>
       </x:c>
       <x:c r="C17" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -888,8 +888,8 @@
       <x:c r="A18" s="41" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B18" s="42" t="n">
-        <x:v>46305.13888888889</x:v>
+      <x:c r="B18" s="35" t="n">
+        <x:v>46299.086805555555</x:v>
       </x:c>
       <x:c r="C18" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -919,7 +919,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B19" s="32" t="n">
-        <x:v>46306.083333333336</x:v>
+        <x:v>46299.163194444445</x:v>
       </x:c>
       <x:c r="C19" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -948,8 +948,8 @@
       <x:c r="A20" s="41" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B20" s="42" t="n">
-        <x:v>46307.145833333336</x:v>
+      <x:c r="B20" s="35" t="n">
+        <x:v>46300.125</x:v>
       </x:c>
       <x:c r="C20" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -979,7 +979,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B21" s="32" t="n">
-        <x:v>46308.083333333336</x:v>
+        <x:v>46300.19097222222</x:v>
       </x:c>
       <x:c r="C21" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1008,8 +1008,8 @@
       <x:c r="A22" s="41" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B22" s="42" t="n">
-        <x:v>46309.15625</x:v>
+      <x:c r="B22" s="35" t="n">
+        <x:v>46301.10763888889</x:v>
       </x:c>
       <x:c r="C22" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1039,7 +1039,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B23" s="32" t="n">
-        <x:v>46310.135416666664</x:v>
+        <x:v>46301.17013888889</x:v>
       </x:c>
       <x:c r="C23" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1068,8 +1068,8 @@
       <x:c r="A24" s="41" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B24" s="42" t="n">
-        <x:v>46311.131944444445</x:v>
+      <x:c r="B24" s="35" t="n">
+        <x:v>46302.09722222222</x:v>
       </x:c>
       <x:c r="C24" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1099,7 +1099,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B25" s="32" t="n">
-        <x:v>46312.18402777778</x:v>
+        <x:v>46302.15625</x:v>
       </x:c>
       <x:c r="C25" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1128,8 +1128,8 @@
       <x:c r="A26" s="41" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B26" s="42" t="n">
-        <x:v>46313.083333333336</x:v>
+      <x:c r="B26" s="35" t="n">
+        <x:v>46303.09027777778</x:v>
       </x:c>
       <x:c r="C26" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1159,7 +1159,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B27" s="32" t="n">
-        <x:v>46314.10763888889</x:v>
+        <x:v>46303.17361111111</x:v>
       </x:c>
       <x:c r="C27" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1188,8 +1188,8 @@
       <x:c r="A28" s="41" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B28" s="42" t="n">
-        <x:v>46315.125</x:v>
+      <x:c r="B28" s="35" t="n">
+        <x:v>46304.11111111111</x:v>
       </x:c>
       <x:c r="C28" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1219,7 +1219,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B29" s="32" t="n">
-        <x:v>46316.194444444445</x:v>
+        <x:v>46304.197916666664</x:v>
       </x:c>
       <x:c r="C29" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1248,8 +1248,8 @@
       <x:c r="A30" s="41" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B30" s="42" t="n">
-        <x:v>46317.13888888889</x:v>
+      <x:c r="B30" s="35" t="n">
+        <x:v>46305.118055555555</x:v>
       </x:c>
       <x:c r="C30" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1279,7 +1279,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B31" s="32" t="n">
-        <x:v>46318.208333333336</x:v>
+        <x:v>46305.1875</x:v>
       </x:c>
       <x:c r="C31" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1308,8 +1308,8 @@
       <x:c r="A32" s="41" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B32" s="42" t="n">
-        <x:v>46319.17361111111</x:v>
+      <x:c r="B32" s="35" t="n">
+        <x:v>46306.09375</x:v>
       </x:c>
       <x:c r="C32" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1339,7 +1339,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B33" s="32" t="n">
-        <x:v>46320.15277777778</x:v>
+        <x:v>46306.19097222222</x:v>
       </x:c>
       <x:c r="C33" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1368,8 +1368,8 @@
       <x:c r="A34" s="41" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B34" s="42" t="n">
-        <x:v>46321.125</x:v>
+      <x:c r="B34" s="35" t="n">
+        <x:v>46307.083333333336</x:v>
       </x:c>
       <x:c r="C34" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1399,7 +1399,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B35" s="32" t="n">
-        <x:v>46322.131944444445</x:v>
+        <x:v>46307.20486111111</x:v>
       </x:c>
       <x:c r="C35" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1428,8 +1428,8 @@
       <x:c r="A36" s="41" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B36" s="42" t="n">
-        <x:v>46323.131944444445</x:v>
+      <x:c r="B36" s="35" t="n">
+        <x:v>46308.11111111111</x:v>
       </x:c>
       <x:c r="C36" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1459,7 +1459,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B37" s="32" t="n">
-        <x:v>46324.177083333336</x:v>
+        <x:v>46308.163194444445</x:v>
       </x:c>
       <x:c r="C37" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1488,8 +1488,8 @@
       <x:c r="A38" s="41" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B38" s="42" t="n">
-        <x:v>46325.19097222222</x:v>
+      <x:c r="B38" s="35" t="n">
+        <x:v>46309.11111111111</x:v>
       </x:c>
       <x:c r="C38" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1519,7 +1519,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B39" s="32" t="n">
-        <x:v>46326.180555555555</x:v>
+        <x:v>46309.20486111111</x:v>
       </x:c>
       <x:c r="C39" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1548,8 +1548,8 @@
       <x:c r="A40" s="41" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B40" s="42" t="n">
-        <x:v>46327.086805555555</x:v>
+      <x:c r="B40" s="35" t="n">
+        <x:v>46310.086805555555</x:v>
       </x:c>
       <x:c r="C40" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1579,7 +1579,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B41" s="32" t="n">
-        <x:v>46328.09722222222</x:v>
+        <x:v>46310.17013888889</x:v>
       </x:c>
       <x:c r="C41" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1608,8 +1608,8 @@
       <x:c r="A42" s="41" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B42" s="42" t="n">
-        <x:v>46329.100694444445</x:v>
+      <x:c r="B42" s="35" t="n">
+        <x:v>46311.09375</x:v>
       </x:c>
       <x:c r="C42" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B43" s="32" t="n">
-        <x:v>46330.145833333336</x:v>
+        <x:v>46311.1875</x:v>
       </x:c>
       <x:c r="C43" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1668,8 +1668,8 @@
       <x:c r="A44" s="41" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B44" s="42" t="n">
-        <x:v>46331.18402777778</x:v>
+      <x:c r="B44" s="35" t="n">
+        <x:v>46312.125</x:v>
       </x:c>
       <x:c r="C44" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1699,7 +1699,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B45" s="32" t="n">
-        <x:v>46332.114583333336</x:v>
+        <x:v>46312.177083333336</x:v>
       </x:c>
       <x:c r="C45" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1728,8 +1728,8 @@
       <x:c r="A46" s="41" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="B46" s="42" t="n">
-        <x:v>46333.145833333336</x:v>
+      <x:c r="B46" s="35" t="n">
+        <x:v>46313.086805555555</x:v>
       </x:c>
       <x:c r="C46" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B47" s="32" t="n">
-        <x:v>46334.12152777778</x:v>
+        <x:v>46313.177083333336</x:v>
       </x:c>
       <x:c r="C47" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1788,8 +1788,8 @@
       <x:c r="A48" s="41" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="B48" s="42" t="n">
-        <x:v>46335.18402777778</x:v>
+      <x:c r="B48" s="35" t="n">
+        <x:v>46314.086805555555</x:v>
       </x:c>
       <x:c r="C48" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1819,7 +1819,7 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B49" s="32" t="n">
-        <x:v>46336.177083333336</x:v>
+        <x:v>46314.15625</x:v>
       </x:c>
       <x:c r="C49" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1848,8 +1848,8 @@
       <x:c r="A50" s="41" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B50" s="42" t="n">
-        <x:v>46337.163194444445</x:v>
+      <x:c r="B50" s="35" t="n">
+        <x:v>46315.114583333336</x:v>
       </x:c>
       <x:c r="C50" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1879,7 +1879,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B51" s="32" t="n">
-        <x:v>46338.11111111111</x:v>
+        <x:v>46315.15625</x:v>
       </x:c>
       <x:c r="C51" s="33" t="str">
         <x:v>New research (existing)</x:v>
@@ -1908,8 +1908,8 @@
       <x:c r="A52" s="41" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B52" s="42" t="n">
-        <x:v>46339.177083333336</x:v>
+      <x:c r="B52" s="35" t="n">
+        <x:v>46316.12152777778</x:v>
       </x:c>
       <x:c r="C52" s="43" t="str">
         <x:v>New research (added)</x:v>
@@ -1936,7 +1936,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca69a94e254a49f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9110f6b6134d5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>